<commit_message>
Canevas : élargir les listes déroulantes agents (A4:A203 / C4:C203) pour couvrir tous les agents d'un poste
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -556,7 +556,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -571,7 +570,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
@@ -621,7 +619,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
@@ -657,7 +654,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
@@ -700,7 +696,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
@@ -913,10 +908,10 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B9 B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$C$4:$C$23</formula1>
+      <formula1>Referentiels!$C$4:$C$203</formula1>
     </dataValidation>
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$A$4:$A$23</formula1>
+      <formula1>Referentiels!$A$4:$A$203</formula1>
     </dataValidation>
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$E$4:$E$13</formula1>
@@ -1948,10 +1943,10 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$A$4:$A$23</formula1>
+      <formula1>Referentiels!$A$4:$A$203</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$C$4:$C$23</formula1>
+      <formula1>Referentiels!$C$4:$C$203</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H300 I2:I300 J2:J300 K2:K300 L2:L300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>

</xml_diff>

<commit_message>
Canevas — listes d'agents par rôle : saisisseur & traitant = membres ; attributaire via feuille « Agents TPR » (agents créés à l'import) ; renommage installateur→traitant
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-Imprimantes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-Switchs et AP" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-Scanners chèque" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referentiels" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agents TPR" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referentiels" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -245,6 +246,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>App</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Agents du poste. Pré-rempli par l'application. Ajoutez ici tout agent attributaire absent de la base ; il sera créé à l'import.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -906,15 +922,18 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="B9 B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$C$4:$C$203</formula1>
-    </dataValidation>
+  <dataValidations count="4">
     <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$A$4:$A$203</formula1>
     </dataValidation>
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$E$4:$E$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Referentiels!$C$4:$C$203</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Referentiels!$G$4:$G$203</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1351,7 +1370,7 @@
       </c>
       <c r="G1" s="10" t="inlineStr">
         <is>
-          <t>Agent installateur *</t>
+          <t>Agent traitant *</t>
         </is>
       </c>
       <c r="H1" s="10" t="inlineStr">
@@ -1943,10 +1962,10 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$A$4:$A$203</formula1>
+      <formula1>'Agents TPR'!$A$2:$A$203</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$C$4:$C$203</formula1>
+      <formula1>Referentiels!$G$4:$G$203</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H300 I2:I300 J2:J300 K2:K300 L2:L300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
@@ -2997,7 +3016,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Matricule *</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Nom *</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Prénom *</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Fonction</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Téléphone</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AG001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DIOP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Awa</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Caissier</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AG002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NDIAYE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Modou</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Comptable</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3005,6 +3123,7 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3037,6 +3156,11 @@
           <t>Catégories de câble</t>
         </is>
       </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Membres de la mission (matricule — nom)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -3054,6 +3178,11 @@
           <t>Cat5e</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>IN001 — SOW Cheikh</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -3069,6 +3198,11 @@
       <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Cat6</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>IN002 — BA Fatou</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Canevas : attributaire affiché « matricule — prénom nom » (colonne libellé auto) ; libelle() en prénom nom ; recalcul forcé
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -1328,8 +1328,8 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -1962,7 +1962,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Agents TPR'!$A$2:$A$203</formula1>
+      <formula1>'Agents TPR'!$H$2:$H$203</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$G$4:$G$203</formula1>
@@ -3016,7 +3016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:H203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3025,6 +3025,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3058,6 +3059,11 @@
           <t>Email</t>
         </is>
       </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>Sélection (auto — ne pas modifier)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3080,6 +3086,10 @@
           <t>Caissier</t>
         </is>
       </c>
+      <c r="H2">
+        <f>IF($A2="","",$A2&amp;" — "&amp;$C2&amp;" "&amp;$B2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3101,6 +3111,1210 @@
         <is>
           <t>Comptable</t>
         </is>
+      </c>
+      <c r="H3">
+        <f>IF($A3="","",$A3&amp;" — "&amp;$C3&amp;" "&amp;$B3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="H4">
+        <f>IF($A4="","",$A4&amp;" — "&amp;$C4&amp;" "&amp;$B4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="H5">
+        <f>IF($A5="","",$A5&amp;" — "&amp;$C5&amp;" "&amp;$B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="H6">
+        <f>IF($A6="","",$A6&amp;" — "&amp;$C6&amp;" "&amp;$B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="H7">
+        <f>IF($A7="","",$A7&amp;" — "&amp;$C7&amp;" "&amp;$B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="H8">
+        <f>IF($A8="","",$A8&amp;" — "&amp;$C8&amp;" "&amp;$B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="H9">
+        <f>IF($A9="","",$A9&amp;" — "&amp;$C9&amp;" "&amp;$B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="H10">
+        <f>IF($A10="","",$A10&amp;" — "&amp;$C10&amp;" "&amp;$B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="H11">
+        <f>IF($A11="","",$A11&amp;" — "&amp;$C11&amp;" "&amp;$B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="H12">
+        <f>IF($A12="","",$A12&amp;" — "&amp;$C12&amp;" "&amp;$B12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="H13">
+        <f>IF($A13="","",$A13&amp;" — "&amp;$C13&amp;" "&amp;$B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="H14">
+        <f>IF($A14="","",$A14&amp;" — "&amp;$C14&amp;" "&amp;$B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="H15">
+        <f>IF($A15="","",$A15&amp;" — "&amp;$C15&amp;" "&amp;$B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16">
+        <f>IF($A16="","",$A16&amp;" — "&amp;$C16&amp;" "&amp;$B16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="H17">
+        <f>IF($A17="","",$A17&amp;" — "&amp;$C17&amp;" "&amp;$B17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="H18">
+        <f>IF($A18="","",$A18&amp;" — "&amp;$C18&amp;" "&amp;$B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="H19">
+        <f>IF($A19="","",$A19&amp;" — "&amp;$C19&amp;" "&amp;$B19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="H20">
+        <f>IF($A20="","",$A20&amp;" — "&amp;$C20&amp;" "&amp;$B20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="H21">
+        <f>IF($A21="","",$A21&amp;" — "&amp;$C21&amp;" "&amp;$B21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="H22">
+        <f>IF($A22="","",$A22&amp;" — "&amp;$C22&amp;" "&amp;$B22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="H23">
+        <f>IF($A23="","",$A23&amp;" — "&amp;$C23&amp;" "&amp;$B23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="H24">
+        <f>IF($A24="","",$A24&amp;" — "&amp;$C24&amp;" "&amp;$B24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="H25">
+        <f>IF($A25="","",$A25&amp;" — "&amp;$C25&amp;" "&amp;$B25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="H26">
+        <f>IF($A26="","",$A26&amp;" — "&amp;$C26&amp;" "&amp;$B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="H27">
+        <f>IF($A27="","",$A27&amp;" — "&amp;$C27&amp;" "&amp;$B27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="H28">
+        <f>IF($A28="","",$A28&amp;" — "&amp;$C28&amp;" "&amp;$B28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="H29">
+        <f>IF($A29="","",$A29&amp;" — "&amp;$C29&amp;" "&amp;$B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30">
+        <f>IF($A30="","",$A30&amp;" — "&amp;$C30&amp;" "&amp;$B30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31">
+        <f>IF($A31="","",$A31&amp;" — "&amp;$C31&amp;" "&amp;$B31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32">
+        <f>IF($A32="","",$A32&amp;" — "&amp;$C32&amp;" "&amp;$B32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="H33">
+        <f>IF($A33="","",$A33&amp;" — "&amp;$C33&amp;" "&amp;$B33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34">
+        <f>IF($A34="","",$A34&amp;" — "&amp;$C34&amp;" "&amp;$B34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="H35">
+        <f>IF($A35="","",$A35&amp;" — "&amp;$C35&amp;" "&amp;$B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="H36">
+        <f>IF($A36="","",$A36&amp;" — "&amp;$C36&amp;" "&amp;$B36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="H37">
+        <f>IF($A37="","",$A37&amp;" — "&amp;$C37&amp;" "&amp;$B37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="H38">
+        <f>IF($A38="","",$A38&amp;" — "&amp;$C38&amp;" "&amp;$B38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="H39">
+        <f>IF($A39="","",$A39&amp;" — "&amp;$C39&amp;" "&amp;$B39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="H40">
+        <f>IF($A40="","",$A40&amp;" — "&amp;$C40&amp;" "&amp;$B40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="H41">
+        <f>IF($A41="","",$A41&amp;" — "&amp;$C41&amp;" "&amp;$B41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42">
+        <f>IF($A42="","",$A42&amp;" — "&amp;$C42&amp;" "&amp;$B42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43">
+        <f>IF($A43="","",$A43&amp;" — "&amp;$C43&amp;" "&amp;$B43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44">
+        <f>IF($A44="","",$A44&amp;" — "&amp;$C44&amp;" "&amp;$B44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45">
+        <f>IF($A45="","",$A45&amp;" — "&amp;$C45&amp;" "&amp;$B45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="H46">
+        <f>IF($A46="","",$A46&amp;" — "&amp;$C46&amp;" "&amp;$B46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="H47">
+        <f>IF($A47="","",$A47&amp;" — "&amp;$C47&amp;" "&amp;$B47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="H48">
+        <f>IF($A48="","",$A48&amp;" — "&amp;$C48&amp;" "&amp;$B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="H49">
+        <f>IF($A49="","",$A49&amp;" — "&amp;$C49&amp;" "&amp;$B49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="H50">
+        <f>IF($A50="","",$A50&amp;" — "&amp;$C50&amp;" "&amp;$B50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="H51">
+        <f>IF($A51="","",$A51&amp;" — "&amp;$C51&amp;" "&amp;$B51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="H52">
+        <f>IF($A52="","",$A52&amp;" — "&amp;$C52&amp;" "&amp;$B52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="H53">
+        <f>IF($A53="","",$A53&amp;" — "&amp;$C53&amp;" "&amp;$B53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="H54">
+        <f>IF($A54="","",$A54&amp;" — "&amp;$C54&amp;" "&amp;$B54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55">
+        <f>IF($A55="","",$A55&amp;" — "&amp;$C55&amp;" "&amp;$B55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="H56">
+        <f>IF($A56="","",$A56&amp;" — "&amp;$C56&amp;" "&amp;$B56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="H57">
+        <f>IF($A57="","",$A57&amp;" — "&amp;$C57&amp;" "&amp;$B57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="H58">
+        <f>IF($A58="","",$A58&amp;" — "&amp;$C58&amp;" "&amp;$B58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59">
+        <f>IF($A59="","",$A59&amp;" — "&amp;$C59&amp;" "&amp;$B59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60">
+        <f>IF($A60="","",$A60&amp;" — "&amp;$C60&amp;" "&amp;$B60)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61">
+        <f>IF($A61="","",$A61&amp;" — "&amp;$C61&amp;" "&amp;$B61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62">
+        <f>IF($A62="","",$A62&amp;" — "&amp;$C62&amp;" "&amp;$B62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63">
+        <f>IF($A63="","",$A63&amp;" — "&amp;$C63&amp;" "&amp;$B63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="H64">
+        <f>IF($A64="","",$A64&amp;" — "&amp;$C64&amp;" "&amp;$B64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="H65">
+        <f>IF($A65="","",$A65&amp;" — "&amp;$C65&amp;" "&amp;$B65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="H66">
+        <f>IF($A66="","",$A66&amp;" — "&amp;$C66&amp;" "&amp;$B66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67">
+        <f>IF($A67="","",$A67&amp;" — "&amp;$C67&amp;" "&amp;$B67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68">
+        <f>IF($A68="","",$A68&amp;" — "&amp;$C68&amp;" "&amp;$B68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69">
+        <f>IF($A69="","",$A69&amp;" — "&amp;$C69&amp;" "&amp;$B69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70">
+        <f>IF($A70="","",$A70&amp;" — "&amp;$C70&amp;" "&amp;$B70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71">
+        <f>IF($A71="","",$A71&amp;" — "&amp;$C71&amp;" "&amp;$B71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72">
+        <f>IF($A72="","",$A72&amp;" — "&amp;$C72&amp;" "&amp;$B72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="H73">
+        <f>IF($A73="","",$A73&amp;" — "&amp;$C73&amp;" "&amp;$B73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="H74">
+        <f>IF($A74="","",$A74&amp;" — "&amp;$C74&amp;" "&amp;$B74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="H75">
+        <f>IF($A75="","",$A75&amp;" — "&amp;$C75&amp;" "&amp;$B75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="H76">
+        <f>IF($A76="","",$A76&amp;" — "&amp;$C76&amp;" "&amp;$B76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="H77">
+        <f>IF($A77="","",$A77&amp;" — "&amp;$C77&amp;" "&amp;$B77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="H78">
+        <f>IF($A78="","",$A78&amp;" — "&amp;$C78&amp;" "&amp;$B78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="H79">
+        <f>IF($A79="","",$A79&amp;" — "&amp;$C79&amp;" "&amp;$B79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="H80">
+        <f>IF($A80="","",$A80&amp;" — "&amp;$C80&amp;" "&amp;$B80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="H81">
+        <f>IF($A81="","",$A81&amp;" — "&amp;$C81&amp;" "&amp;$B81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="H82">
+        <f>IF($A82="","",$A82&amp;" — "&amp;$C82&amp;" "&amp;$B82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="H83">
+        <f>IF($A83="","",$A83&amp;" — "&amp;$C83&amp;" "&amp;$B83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="H84">
+        <f>IF($A84="","",$A84&amp;" — "&amp;$C84&amp;" "&amp;$B84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="H85">
+        <f>IF($A85="","",$A85&amp;" — "&amp;$C85&amp;" "&amp;$B85)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="H86">
+        <f>IF($A86="","",$A86&amp;" — "&amp;$C86&amp;" "&amp;$B86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="H87">
+        <f>IF($A87="","",$A87&amp;" — "&amp;$C87&amp;" "&amp;$B87)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="H88">
+        <f>IF($A88="","",$A88&amp;" — "&amp;$C88&amp;" "&amp;$B88)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="H89">
+        <f>IF($A89="","",$A89&amp;" — "&amp;$C89&amp;" "&amp;$B89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="H90">
+        <f>IF($A90="","",$A90&amp;" — "&amp;$C90&amp;" "&amp;$B90)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="H91">
+        <f>IF($A91="","",$A91&amp;" — "&amp;$C91&amp;" "&amp;$B91)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="H92">
+        <f>IF($A92="","",$A92&amp;" — "&amp;$C92&amp;" "&amp;$B92)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="H93">
+        <f>IF($A93="","",$A93&amp;" — "&amp;$C93&amp;" "&amp;$B93)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="H94">
+        <f>IF($A94="","",$A94&amp;" — "&amp;$C94&amp;" "&amp;$B94)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="H95">
+        <f>IF($A95="","",$A95&amp;" — "&amp;$C95&amp;" "&amp;$B95)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="H96">
+        <f>IF($A96="","",$A96&amp;" — "&amp;$C96&amp;" "&amp;$B96)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="H97">
+        <f>IF($A97="","",$A97&amp;" — "&amp;$C97&amp;" "&amp;$B97)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="H98">
+        <f>IF($A98="","",$A98&amp;" — "&amp;$C98&amp;" "&amp;$B98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="H99">
+        <f>IF($A99="","",$A99&amp;" — "&amp;$C99&amp;" "&amp;$B99)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="H100">
+        <f>IF($A100="","",$A100&amp;" — "&amp;$C100&amp;" "&amp;$B100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="H101">
+        <f>IF($A101="","",$A101&amp;" — "&amp;$C101&amp;" "&amp;$B101)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="H102">
+        <f>IF($A102="","",$A102&amp;" — "&amp;$C102&amp;" "&amp;$B102)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="H103">
+        <f>IF($A103="","",$A103&amp;" — "&amp;$C103&amp;" "&amp;$B103)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="H104">
+        <f>IF($A104="","",$A104&amp;" — "&amp;$C104&amp;" "&amp;$B104)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="H105">
+        <f>IF($A105="","",$A105&amp;" — "&amp;$C105&amp;" "&amp;$B105)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="H106">
+        <f>IF($A106="","",$A106&amp;" — "&amp;$C106&amp;" "&amp;$B106)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="H107">
+        <f>IF($A107="","",$A107&amp;" — "&amp;$C107&amp;" "&amp;$B107)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="H108">
+        <f>IF($A108="","",$A108&amp;" — "&amp;$C108&amp;" "&amp;$B108)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="H109">
+        <f>IF($A109="","",$A109&amp;" — "&amp;$C109&amp;" "&amp;$B109)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="H110">
+        <f>IF($A110="","",$A110&amp;" — "&amp;$C110&amp;" "&amp;$B110)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="H111">
+        <f>IF($A111="","",$A111&amp;" — "&amp;$C111&amp;" "&amp;$B111)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="H112">
+        <f>IF($A112="","",$A112&amp;" — "&amp;$C112&amp;" "&amp;$B112)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="H113">
+        <f>IF($A113="","",$A113&amp;" — "&amp;$C113&amp;" "&amp;$B113)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="H114">
+        <f>IF($A114="","",$A114&amp;" — "&amp;$C114&amp;" "&amp;$B114)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="H115">
+        <f>IF($A115="","",$A115&amp;" — "&amp;$C115&amp;" "&amp;$B115)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="H116">
+        <f>IF($A116="","",$A116&amp;" — "&amp;$C116&amp;" "&amp;$B116)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="H117">
+        <f>IF($A117="","",$A117&amp;" — "&amp;$C117&amp;" "&amp;$B117)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="H118">
+        <f>IF($A118="","",$A118&amp;" — "&amp;$C118&amp;" "&amp;$B118)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="H119">
+        <f>IF($A119="","",$A119&amp;" — "&amp;$C119&amp;" "&amp;$B119)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="H120">
+        <f>IF($A120="","",$A120&amp;" — "&amp;$C120&amp;" "&amp;$B120)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="H121">
+        <f>IF($A121="","",$A121&amp;" — "&amp;$C121&amp;" "&amp;$B121)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="H122">
+        <f>IF($A122="","",$A122&amp;" — "&amp;$C122&amp;" "&amp;$B122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="H123">
+        <f>IF($A123="","",$A123&amp;" — "&amp;$C123&amp;" "&amp;$B123)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="H124">
+        <f>IF($A124="","",$A124&amp;" — "&amp;$C124&amp;" "&amp;$B124)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="H125">
+        <f>IF($A125="","",$A125&amp;" — "&amp;$C125&amp;" "&amp;$B125)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="H126">
+        <f>IF($A126="","",$A126&amp;" — "&amp;$C126&amp;" "&amp;$B126)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="H127">
+        <f>IF($A127="","",$A127&amp;" — "&amp;$C127&amp;" "&amp;$B127)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="H128">
+        <f>IF($A128="","",$A128&amp;" — "&amp;$C128&amp;" "&amp;$B128)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="H129">
+        <f>IF($A129="","",$A129&amp;" — "&amp;$C129&amp;" "&amp;$B129)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="H130">
+        <f>IF($A130="","",$A130&amp;" — "&amp;$C130&amp;" "&amp;$B130)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="H131">
+        <f>IF($A131="","",$A131&amp;" — "&amp;$C131&amp;" "&amp;$B131)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="H132">
+        <f>IF($A132="","",$A132&amp;" — "&amp;$C132&amp;" "&amp;$B132)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="H133">
+        <f>IF($A133="","",$A133&amp;" — "&amp;$C133&amp;" "&amp;$B133)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="H134">
+        <f>IF($A134="","",$A134&amp;" — "&amp;$C134&amp;" "&amp;$B134)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="H135">
+        <f>IF($A135="","",$A135&amp;" — "&amp;$C135&amp;" "&amp;$B135)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="H136">
+        <f>IF($A136="","",$A136&amp;" — "&amp;$C136&amp;" "&amp;$B136)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="H137">
+        <f>IF($A137="","",$A137&amp;" — "&amp;$C137&amp;" "&amp;$B137)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="H138">
+        <f>IF($A138="","",$A138&amp;" — "&amp;$C138&amp;" "&amp;$B138)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="H139">
+        <f>IF($A139="","",$A139&amp;" — "&amp;$C139&amp;" "&amp;$B139)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="H140">
+        <f>IF($A140="","",$A140&amp;" — "&amp;$C140&amp;" "&amp;$B140)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="H141">
+        <f>IF($A141="","",$A141&amp;" — "&amp;$C141&amp;" "&amp;$B141)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="H142">
+        <f>IF($A142="","",$A142&amp;" — "&amp;$C142&amp;" "&amp;$B142)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="H143">
+        <f>IF($A143="","",$A143&amp;" — "&amp;$C143&amp;" "&amp;$B143)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="H144">
+        <f>IF($A144="","",$A144&amp;" — "&amp;$C144&amp;" "&amp;$B144)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="H145">
+        <f>IF($A145="","",$A145&amp;" — "&amp;$C145&amp;" "&amp;$B145)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="H146">
+        <f>IF($A146="","",$A146&amp;" — "&amp;$C146&amp;" "&amp;$B146)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="H147">
+        <f>IF($A147="","",$A147&amp;" — "&amp;$C147&amp;" "&amp;$B147)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="H148">
+        <f>IF($A148="","",$A148&amp;" — "&amp;$C148&amp;" "&amp;$B148)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="H149">
+        <f>IF($A149="","",$A149&amp;" — "&amp;$C149&amp;" "&amp;$B149)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="H150">
+        <f>IF($A150="","",$A150&amp;" — "&amp;$C150&amp;" "&amp;$B150)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="H151">
+        <f>IF($A151="","",$A151&amp;" — "&amp;$C151&amp;" "&amp;$B151)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="H152">
+        <f>IF($A152="","",$A152&amp;" — "&amp;$C152&amp;" "&amp;$B152)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="H153">
+        <f>IF($A153="","",$A153&amp;" — "&amp;$C153&amp;" "&amp;$B153)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="H154">
+        <f>IF($A154="","",$A154&amp;" — "&amp;$C154&amp;" "&amp;$B154)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="H155">
+        <f>IF($A155="","",$A155&amp;" — "&amp;$C155&amp;" "&amp;$B155)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="H156">
+        <f>IF($A156="","",$A156&amp;" — "&amp;$C156&amp;" "&amp;$B156)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="H157">
+        <f>IF($A157="","",$A157&amp;" — "&amp;$C157&amp;" "&amp;$B157)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="H158">
+        <f>IF($A158="","",$A158&amp;" — "&amp;$C158&amp;" "&amp;$B158)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="H159">
+        <f>IF($A159="","",$A159&amp;" — "&amp;$C159&amp;" "&amp;$B159)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="H160">
+        <f>IF($A160="","",$A160&amp;" — "&amp;$C160&amp;" "&amp;$B160)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="H161">
+        <f>IF($A161="","",$A161&amp;" — "&amp;$C161&amp;" "&amp;$B161)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="H162">
+        <f>IF($A162="","",$A162&amp;" — "&amp;$C162&amp;" "&amp;$B162)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="H163">
+        <f>IF($A163="","",$A163&amp;" — "&amp;$C163&amp;" "&amp;$B163)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="H164">
+        <f>IF($A164="","",$A164&amp;" — "&amp;$C164&amp;" "&amp;$B164)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="H165">
+        <f>IF($A165="","",$A165&amp;" — "&amp;$C165&amp;" "&amp;$B165)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="H166">
+        <f>IF($A166="","",$A166&amp;" — "&amp;$C166&amp;" "&amp;$B166)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="H167">
+        <f>IF($A167="","",$A167&amp;" — "&amp;$C167&amp;" "&amp;$B167)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="H168">
+        <f>IF($A168="","",$A168&amp;" — "&amp;$C168&amp;" "&amp;$B168)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="H169">
+        <f>IF($A169="","",$A169&amp;" — "&amp;$C169&amp;" "&amp;$B169)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="H170">
+        <f>IF($A170="","",$A170&amp;" — "&amp;$C170&amp;" "&amp;$B170)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="H171">
+        <f>IF($A171="","",$A171&amp;" — "&amp;$C171&amp;" "&amp;$B171)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="H172">
+        <f>IF($A172="","",$A172&amp;" — "&amp;$C172&amp;" "&amp;$B172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="H173">
+        <f>IF($A173="","",$A173&amp;" — "&amp;$C173&amp;" "&amp;$B173)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="H174">
+        <f>IF($A174="","",$A174&amp;" — "&amp;$C174&amp;" "&amp;$B174)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="H175">
+        <f>IF($A175="","",$A175&amp;" — "&amp;$C175&amp;" "&amp;$B175)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="H176">
+        <f>IF($A176="","",$A176&amp;" — "&amp;$C176&amp;" "&amp;$B176)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="H177">
+        <f>IF($A177="","",$A177&amp;" — "&amp;$C177&amp;" "&amp;$B177)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="H178">
+        <f>IF($A178="","",$A178&amp;" — "&amp;$C178&amp;" "&amp;$B178)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="H179">
+        <f>IF($A179="","",$A179&amp;" — "&amp;$C179&amp;" "&amp;$B179)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="H180">
+        <f>IF($A180="","",$A180&amp;" — "&amp;$C180&amp;" "&amp;$B180)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="H181">
+        <f>IF($A181="","",$A181&amp;" — "&amp;$C181&amp;" "&amp;$B181)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="H182">
+        <f>IF($A182="","",$A182&amp;" — "&amp;$C182&amp;" "&amp;$B182)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="H183">
+        <f>IF($A183="","",$A183&amp;" — "&amp;$C183&amp;" "&amp;$B183)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="H184">
+        <f>IF($A184="","",$A184&amp;" — "&amp;$C184&amp;" "&amp;$B184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="H185">
+        <f>IF($A185="","",$A185&amp;" — "&amp;$C185&amp;" "&amp;$B185)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="H186">
+        <f>IF($A186="","",$A186&amp;" — "&amp;$C186&amp;" "&amp;$B186)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="H187">
+        <f>IF($A187="","",$A187&amp;" — "&amp;$C187&amp;" "&amp;$B187)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="H188">
+        <f>IF($A188="","",$A188&amp;" — "&amp;$C188&amp;" "&amp;$B188)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="H189">
+        <f>IF($A189="","",$A189&amp;" — "&amp;$C189&amp;" "&amp;$B189)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="H190">
+        <f>IF($A190="","",$A190&amp;" — "&amp;$C190&amp;" "&amp;$B190)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="H191">
+        <f>IF($A191="","",$A191&amp;" — "&amp;$C191&amp;" "&amp;$B191)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="H192">
+        <f>IF($A192="","",$A192&amp;" — "&amp;$C192&amp;" "&amp;$B192)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="H193">
+        <f>IF($A193="","",$A193&amp;" — "&amp;$C193&amp;" "&amp;$B193)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="H194">
+        <f>IF($A194="","",$A194&amp;" — "&amp;$C194&amp;" "&amp;$B194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="H195">
+        <f>IF($A195="","",$A195&amp;" — "&amp;$C195&amp;" "&amp;$B195)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="H196">
+        <f>IF($A196="","",$A196&amp;" — "&amp;$C196&amp;" "&amp;$B196)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="H197">
+        <f>IF($A197="","",$A197&amp;" — "&amp;$C197&amp;" "&amp;$B197)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="H198">
+        <f>IF($A198="","",$A198&amp;" — "&amp;$C198&amp;" "&amp;$B198)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="H199">
+        <f>IF($A199="","",$A199&amp;" — "&amp;$C199&amp;" "&amp;$B199)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="H200">
+        <f>IF($A200="","",$A200&amp;" — "&amp;$C200&amp;" "&amp;$B200)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="H201">
+        <f>IF($A201="","",$A201&amp;" — "&amp;$C201&amp;" "&amp;$B201)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="H202">
+        <f>IF($A202="","",$A202&amp;" — "&amp;$C202&amp;" "&amp;$B202)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="203">
+      <c r="H203">
+        <f>IF($A203="","",$A203&amp;" — "&amp;$C203&amp;" "&amp;$B203)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Canevas : retrait des listes Agents de poste (A) et Informaticiens (C) du référentiel ; référentiel réduit à Membres (A) + Catégories (C) ; chefs sans liste (pré-remplis)
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -922,18 +922,12 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$A$4:$A$203</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$E$4:$E$13</formula1>
-    </dataValidation>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$C$4:$C$203</formula1>
+      <formula1>Referentiels!$C$4:$C$13</formula1>
     </dataValidation>
     <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$G$4:$G$203</formula1>
+      <formula1>Referentiels!$A$4:$A$203</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1965,7 +1959,7 @@
       <formula1>'Agents TPR'!$H$2:$H$203</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Referentiels!$G$4:$G$203</formula1>
+      <formula1>Referentiels!$A$4:$A$203</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H300 I2:I300 J2:J300 K2:K300 L2:L300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
@@ -4329,15 +4323,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4357,100 +4351,270 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Agents de poste (matricule — nom)</t>
+          <t>Membres de la mission (matricule — prénom nom)</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Agents informaticiens (matricule — nom)</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
           <t>Catégories de câble</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>Membres de la mission (matricule — nom)</t>
-        </is>
-      </c>
+      <c r="E3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>AG001 — DIOP Awa</t>
+          <t>IN001 — Cheikh SOW</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>IN001 — SOW Cheikh</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
           <t>Cat5e</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>IN001 — SOW Cheikh</t>
-        </is>
-      </c>
+      <c r="E4" s="14" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>AG002 — NDIAYE Modou</t>
+          <t>IN002 — Fatou BA</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>IN002 — BA Fatou</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
           <t>Cat6</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>IN002 — BA Fatou</t>
-        </is>
-      </c>
+      <c r="E5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>AG003 — FALL Aïssatou</t>
-        </is>
-      </c>
+      <c r="A6" s="14" t="n"/>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>IN003 — SECK Ousmane</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
           <t>Cat6a</t>
         </is>
       </c>
+      <c r="E6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="E7" s="14" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Cat7</t>
         </is>
       </c>
+      <c r="E7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="E8" s="14" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Autre</t>
         </is>
       </c>
-    </row>
+      <c r="E8" s="14" t="n"/>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Canevas : suppression de la mention « Exemples — en production... » du référentiel
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -572,6 +572,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -586,6 +587,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
@@ -635,6 +637,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
@@ -670,6 +673,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
@@ -712,6 +716,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
@@ -766,6 +771,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -4323,7 +4329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H210"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4342,11 +4348,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Exemples — en production, l'application remplit ces listes automatiquement pour le poste concerné.</t>
-        </is>
-      </c>
+      <c r="A2" s="12" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
@@ -4413,208 +4415,6 @@
       </c>
       <c r="E8" s="14" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Canevas : libellé attributaire écrit en valeur (matricule — prénom nom) par l'application + exemples littéraux, pour un affichage fiable sans recalcul
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -572,7 +572,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -587,7 +586,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
@@ -637,7 +635,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
@@ -673,7 +670,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
@@ -716,7 +712,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
@@ -771,7 +766,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -3086,9 +3080,10 @@
           <t>Caissier</t>
         </is>
       </c>
-      <c r="H2">
-        <f>IF($A2="","",$A2&amp;" — "&amp;$C2&amp;" "&amp;$B2)</f>
-        <v/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>AG001 — Awa DIOP</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3112,9 +3107,10 @@
           <t>Comptable</t>
         </is>
       </c>
-      <c r="H3">
-        <f>IF($A3="","",$A3&amp;" — "&amp;$C3&amp;" "&amp;$B3)</f>
-        <v/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AG002 — Modou NDIAYE</t>
+        </is>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Canevas : mise en forme conditionnelle (rouge) sur les champs obligatoires vides
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -176,6 +176,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -766,6 +779,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -922,6 +936,46 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B3)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="0">
+      <formula>ISBLANK(B11)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$C$4:$C$13</formula1>
@@ -1304,6 +1358,21 @@
       <c r="F41" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:A100">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(A2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B100">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C100">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(C2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1954,6 +2023,26 @@
       <c r="L41" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B300">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$L2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D300">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(D2),COUNTA($A2:$L2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F300">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(F2),COUNTA($A2:$L2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G300">
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(G2),COUNTA($A2:$L2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Agents TPR'!$H$2:$H$203</formula1>
@@ -2339,6 +2428,16 @@
       <c r="F41" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B300">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D300">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(D2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2713,6 +2812,21 @@
       <c r="F41" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B300">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C300">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(C2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E300">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(E2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Switch,Access point"</formula1>
@@ -3000,6 +3114,11 @@
       <c r="D41" s="11" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B300">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$D2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4314,6 +4433,21 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:A203">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(A2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B203">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(B2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C203">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>AND(ISBLANK(C2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Canevas : liste attributaire en plage nommée dynamique (que les agents TPR renseignés) + alerte MAC mal formée
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -17,7 +17,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agents TPR" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referentiels" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="ListeAttributaires">OFFSET('Agents TPR'!$H$2,0,0,MAX(1,COUNTA('Agents TPR'!$A$2:$A$203)),1)</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -183,7 +185,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="009C0006"/>
@@ -216,6 +218,17 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
           <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+          <bgColor rgb="00FFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4322,6 +4335,9 @@
     <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(D2),COUNTA($A2:$L2)&gt;0)</formula>
     </cfRule>
+    <cfRule type="expression" priority="5" dxfId="3" stopIfTrue="0">
+      <formula>AND($D2&lt;&gt;"",OR(LEN($D2)&lt;&gt;17,LEN($D2)-LEN(SUBSTITUTE($D2,":",""))&lt;&gt;5))</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F300">
     <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
@@ -4333,9 +4349,14 @@
       <formula>AND(ISBLANK(G2),COUNTA($A2:$L2)&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E300">
+    <cfRule type="expression" priority="6" dxfId="3" stopIfTrue="0">
+      <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Agents TPR'!$H$2:$H$203</formula1>
+      <formula1>ListeAttributaires</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Referentiels!$A$4:$A$203</formula1>
@@ -6447,6 +6468,14 @@
     <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(D2),COUNTA($A2:$F2)&gt;0)</formula>
     </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3" stopIfTrue="0">
+      <formula>AND($D2&lt;&gt;"",OR(LEN($D2)&lt;&gt;17,LEN($D2)-LEN(SUBSTITUTE($D2,":",""))&lt;&gt;5))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E300">
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="0">
+      <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8555,6 +8584,9 @@
   <conditionalFormatting sqref="E2:E300">
     <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(E2),COUNTA($A2:$F2)&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="0">
+      <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Canevas : validation de saisie MAC (format AA:BB:CC:DD:EE:FF imposé + message d'aide) sur tous les champs MAC
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -4354,7 +4354,7 @@
       <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>ListeAttributaires</formula1>
     </dataValidation>
@@ -4363,6 +4363,12 @@
     </dataValidation>
     <dataValidation sqref="H2:H300 I2:I300 J2:J300 K2:K300 L2:L300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Adresse MAC invalide" error="Format attendu : AA:BB:CC:DD:EE:FF — 6 paires hexadécimales (0-9, A-F) séparées par « : »." promptTitle="Format adresse MAC" prompt="6 paires hexadécimales séparées par « : », ex. 00:1A:2B:3C:4D:5E" type="custom" errorStyle="stop">
+      <formula1>AND(LEN(D2)=17,LEN(SUBSTITUTE(D2,":",""))=12,MID(D2,3,1)=":",MID(D2,6,1)=":",MID(D2,9,1)=":",MID(D2,12,1)=":",MID(D2,15,1)=":",ISNUMBER(HEX2DEC(LEFT(SUBSTITUTE(D2,":",""),6))),ISNUMBER(HEX2DEC(MID(SUBSTITUTE(D2,":",""),7,6))))</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Adresse MAC invalide" error="Format attendu : AA:BB:CC:DD:EE:FF — 6 paires hexadécimales (0-9, A-F) séparées par « : »." promptTitle="Format adresse MAC" prompt="6 paires hexadécimales séparées par « : », ex. 00:1A:2B:3C:4D:5E" type="custom" errorStyle="stop">
+      <formula1>AND(LEN(E2)=17,LEN(SUBSTITUTE(E2,":",""))=12,MID(E2,3,1)=":",MID(E2,6,1)=":",MID(E2,9,1)=":",MID(E2,12,1)=":",MID(E2,15,1)=":",ISNUMBER(HEX2DEC(LEFT(SUBSTITUTE(E2,":",""),6))),ISNUMBER(HEX2DEC(MID(SUBSTITUTE(E2,":",""),7,6))))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6477,6 +6483,14 @@
       <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Adresse MAC invalide" error="Format attendu : AA:BB:CC:DD:EE:FF — 6 paires hexadécimales (0-9, A-F) séparées par « : »." promptTitle="Format adresse MAC" prompt="6 paires hexadécimales séparées par « : », ex. 00:1A:2B:3C:4D:5E" type="custom" errorStyle="stop">
+      <formula1>AND(LEN(D2)=17,LEN(SUBSTITUTE(D2,":",""))=12,MID(D2,3,1)=":",MID(D2,6,1)=":",MID(D2,9,1)=":",MID(D2,12,1)=":",MID(D2,15,1)=":",ISNUMBER(HEX2DEC(LEFT(SUBSTITUTE(D2,":",""),6))),ISNUMBER(HEX2DEC(MID(SUBSTITUTE(D2,":",""),7,6))))</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Adresse MAC invalide" error="Format attendu : AA:BB:CC:DD:EE:FF — 6 paires hexadécimales (0-9, A-F) séparées par « : »." promptTitle="Format adresse MAC" prompt="6 paires hexadécimales séparées par « : », ex. 00:1A:2B:3C:4D:5E" type="custom" errorStyle="stop">
+      <formula1>AND(LEN(E2)=17,LEN(SUBSTITUTE(E2,":",""))=12,MID(E2,3,1)=":",MID(E2,6,1)=":",MID(E2,9,1)=":",MID(E2,12,1)=":",MID(E2,15,1)=":",ISNUMBER(HEX2DEC(LEFT(SUBSTITUTE(E2,":",""),6))),ISNUMBER(HEX2DEC(MID(SUBSTITUTE(E2,":",""),7,6))))</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8589,9 +8603,12 @@
       <formula>AND($E2&lt;&gt;"",OR(LEN($E2)&lt;&gt;17,LEN($E2)-LEN(SUBSTITUTE($E2,":",""))&lt;&gt;5))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Switch,Access point"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Adresse MAC invalide" error="Format attendu : AA:BB:CC:DD:EE:FF — 6 paires hexadécimales (0-9, A-F) séparées par « : »." promptTitle="Format adresse MAC" prompt="6 paires hexadécimales séparées par « : », ex. 00:1A:2B:3C:4D:5E" type="custom" errorStyle="stop">
+      <formula1>AND(LEN(E2)=17,LEN(SUBSTITUTE(E2,":",""))=12,MID(E2,3,1)=":",MID(E2,6,1)=":",MID(E2,9,1)=":",MID(E2,12,1)=":",MID(E2,15,1)=":",ISNUMBER(HEX2DEC(LEFT(SUBSTITUTE(E2,":",""),6))),ISNUMBER(HEX2DEC(MID(SUBSTITUTE(E2,":",""),7,6))))</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Canevas : retrait des exemples d'agents (AG001/AG002, IN001/IN002) qui apparaissaient dans les listes
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -10684,30 +10684,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AG001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DIOP</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Awa</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Caissier</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>AG001 — Awa DIOP</t>
-        </is>
+      <c r="H2">
+        <f>IF($A2="","",$A2&amp;" — "&amp;$C2&amp;" "&amp;$B2)</f>
+        <v/>
       </c>
       <c r="J2">
         <f>IF(COUNTA($A2:$F2)=0,0,IF(OR($A2="",$B2="",$C2=""),1,0))</f>
@@ -10715,30 +10694,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AG002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>NDIAYE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Modou</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Comptable</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>AG002 — Modou NDIAYE</t>
-        </is>
+      <c r="H3">
+        <f>IF($A3="","",$A3&amp;" — "&amp;$C3&amp;" "&amp;$B3)</f>
+        <v/>
       </c>
       <c r="J3">
         <f>IF(COUNTA($A3:$F3)=0,0,IF(OR($A3="",$B3="",$C3=""),1,0))</f>
@@ -12808,11 +12766,7 @@
       <c r="G3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>IN001 — Cheikh SOW</t>
-        </is>
-      </c>
+      <c r="A4" s="14" t="n"/>
       <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Cat5e</t>
@@ -12821,11 +12775,7 @@
       <c r="E4" s="14" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>IN002 — Fatou BA</t>
-        </is>
-      </c>
+      <c r="A5" s="14" t="n"/>
       <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Cat6</t>

</xml_diff>

<commit_message>
Canevas : bordures de tableau sur les colonnes ajoutees (RAM, processeur, disque, statut, observations) pour retablir la grille
</commit_message>
<xml_diff>
--- a/src/main/resources/canevas/canevas-vierge.xlsx
+++ b/src/main/resources/canevas/canevas-vierge.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -189,6 +189,9 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -1026,6 +1029,10 @@
         </is>
       </c>
       <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="24" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
@@ -2512,11 +2519,11 @@
       <c r="J2" s="23" t="n"/>
       <c r="K2" s="23" t="n"/>
       <c r="L2" s="23" t="n"/>
-      <c r="M2" s="24" t="n"/>
-      <c r="N2" s="24" t="n"/>
-      <c r="O2" s="24" t="n"/>
-      <c r="P2" s="24" t="n"/>
-      <c r="Q2" s="24" t="n"/>
+      <c r="M2" s="25" t="n"/>
+      <c r="N2" s="25" t="n"/>
+      <c r="O2" s="25" t="n"/>
+      <c r="P2" s="25" t="n"/>
+      <c r="Q2" s="25" t="n"/>
       <c r="S2">
         <f>IF(COUNTA($A2:$Q2)=0,0,IF(OR($B2="",$D2="",$F2="",$G2=""),1,0))</f>
         <v/>
@@ -2539,11 +2546,11 @@
       <c r="J3" s="23" t="n"/>
       <c r="K3" s="23" t="n"/>
       <c r="L3" s="23" t="n"/>
-      <c r="M3" s="24" t="n"/>
-      <c r="N3" s="24" t="n"/>
-      <c r="O3" s="24" t="n"/>
-      <c r="P3" s="24" t="n"/>
-      <c r="Q3" s="24" t="n"/>
+      <c r="M3" s="25" t="n"/>
+      <c r="N3" s="25" t="n"/>
+      <c r="O3" s="25" t="n"/>
+      <c r="P3" s="25" t="n"/>
+      <c r="Q3" s="25" t="n"/>
       <c r="S3">
         <f>IF(COUNTA($A3:$Q3)=0,0,IF(OR($B3="",$D3="",$F3="",$G3=""),1,0))</f>
         <v/>
@@ -2566,11 +2573,11 @@
       <c r="J4" s="23" t="n"/>
       <c r="K4" s="23" t="n"/>
       <c r="L4" s="23" t="n"/>
-      <c r="M4" s="24" t="n"/>
-      <c r="N4" s="24" t="n"/>
-      <c r="O4" s="24" t="n"/>
-      <c r="P4" s="24" t="n"/>
-      <c r="Q4" s="24" t="n"/>
+      <c r="M4" s="25" t="n"/>
+      <c r="N4" s="25" t="n"/>
+      <c r="O4" s="25" t="n"/>
+      <c r="P4" s="25" t="n"/>
+      <c r="Q4" s="25" t="n"/>
       <c r="S4">
         <f>IF(COUNTA($A4:$Q4)=0,0,IF(OR($B4="",$D4="",$F4="",$G4=""),1,0))</f>
         <v/>
@@ -2593,11 +2600,11 @@
       <c r="J5" s="23" t="n"/>
       <c r="K5" s="23" t="n"/>
       <c r="L5" s="23" t="n"/>
-      <c r="M5" s="24" t="n"/>
-      <c r="N5" s="24" t="n"/>
-      <c r="O5" s="24" t="n"/>
-      <c r="P5" s="24" t="n"/>
-      <c r="Q5" s="24" t="n"/>
+      <c r="M5" s="25" t="n"/>
+      <c r="N5" s="25" t="n"/>
+      <c r="O5" s="25" t="n"/>
+      <c r="P5" s="25" t="n"/>
+      <c r="Q5" s="25" t="n"/>
       <c r="S5">
         <f>IF(COUNTA($A5:$Q5)=0,0,IF(OR($B5="",$D5="",$F5="",$G5=""),1,0))</f>
         <v/>
@@ -2620,11 +2627,11 @@
       <c r="J6" s="23" t="n"/>
       <c r="K6" s="23" t="n"/>
       <c r="L6" s="23" t="n"/>
-      <c r="M6" s="24" t="n"/>
-      <c r="N6" s="24" t="n"/>
-      <c r="O6" s="24" t="n"/>
-      <c r="P6" s="24" t="n"/>
-      <c r="Q6" s="24" t="n"/>
+      <c r="M6" s="25" t="n"/>
+      <c r="N6" s="25" t="n"/>
+      <c r="O6" s="25" t="n"/>
+      <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="25" t="n"/>
       <c r="S6">
         <f>IF(COUNTA($A6:$Q6)=0,0,IF(OR($B6="",$D6="",$F6="",$G6=""),1,0))</f>
         <v/>
@@ -2647,11 +2654,11 @@
       <c r="J7" s="23" t="n"/>
       <c r="K7" s="23" t="n"/>
       <c r="L7" s="23" t="n"/>
-      <c r="M7" s="24" t="n"/>
-      <c r="N7" s="24" t="n"/>
-      <c r="O7" s="24" t="n"/>
-      <c r="P7" s="24" t="n"/>
-      <c r="Q7" s="24" t="n"/>
+      <c r="M7" s="25" t="n"/>
+      <c r="N7" s="25" t="n"/>
+      <c r="O7" s="25" t="n"/>
+      <c r="P7" s="25" t="n"/>
+      <c r="Q7" s="25" t="n"/>
       <c r="S7">
         <f>IF(COUNTA($A7:$Q7)=0,0,IF(OR($B7="",$D7="",$F7="",$G7=""),1,0))</f>
         <v/>
@@ -2674,11 +2681,11 @@
       <c r="J8" s="23" t="n"/>
       <c r="K8" s="23" t="n"/>
       <c r="L8" s="23" t="n"/>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="24" t="n"/>
-      <c r="P8" s="24" t="n"/>
-      <c r="Q8" s="24" t="n"/>
+      <c r="M8" s="25" t="n"/>
+      <c r="N8" s="25" t="n"/>
+      <c r="O8" s="25" t="n"/>
+      <c r="P8" s="25" t="n"/>
+      <c r="Q8" s="25" t="n"/>
       <c r="S8">
         <f>IF(COUNTA($A8:$Q8)=0,0,IF(OR($B8="",$D8="",$F8="",$G8=""),1,0))</f>
         <v/>
@@ -2701,11 +2708,11 @@
       <c r="J9" s="23" t="n"/>
       <c r="K9" s="23" t="n"/>
       <c r="L9" s="23" t="n"/>
-      <c r="M9" s="24" t="n"/>
-      <c r="N9" s="24" t="n"/>
-      <c r="O9" s="24" t="n"/>
-      <c r="P9" s="24" t="n"/>
-      <c r="Q9" s="24" t="n"/>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="25" t="n"/>
+      <c r="O9" s="25" t="n"/>
+      <c r="P9" s="25" t="n"/>
+      <c r="Q9" s="25" t="n"/>
       <c r="S9">
         <f>IF(COUNTA($A9:$Q9)=0,0,IF(OR($B9="",$D9="",$F9="",$G9=""),1,0))</f>
         <v/>
@@ -2728,11 +2735,11 @@
       <c r="J10" s="23" t="n"/>
       <c r="K10" s="23" t="n"/>
       <c r="L10" s="23" t="n"/>
-      <c r="M10" s="24" t="n"/>
-      <c r="N10" s="24" t="n"/>
-      <c r="O10" s="24" t="n"/>
-      <c r="P10" s="24" t="n"/>
-      <c r="Q10" s="24" t="n"/>
+      <c r="M10" s="25" t="n"/>
+      <c r="N10" s="25" t="n"/>
+      <c r="O10" s="25" t="n"/>
+      <c r="P10" s="25" t="n"/>
+      <c r="Q10" s="25" t="n"/>
       <c r="S10">
         <f>IF(COUNTA($A10:$Q10)=0,0,IF(OR($B10="",$D10="",$F10="",$G10=""),1,0))</f>
         <v/>
@@ -2755,11 +2762,11 @@
       <c r="J11" s="23" t="n"/>
       <c r="K11" s="23" t="n"/>
       <c r="L11" s="23" t="n"/>
-      <c r="M11" s="24" t="n"/>
-      <c r="N11" s="24" t="n"/>
-      <c r="O11" s="24" t="n"/>
-      <c r="P11" s="24" t="n"/>
-      <c r="Q11" s="24" t="n"/>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="25" t="n"/>
+      <c r="O11" s="25" t="n"/>
+      <c r="P11" s="25" t="n"/>
+      <c r="Q11" s="25" t="n"/>
       <c r="S11">
         <f>IF(COUNTA($A11:$Q11)=0,0,IF(OR($B11="",$D11="",$F11="",$G11=""),1,0))</f>
         <v/>
@@ -2782,11 +2789,11 @@
       <c r="J12" s="23" t="n"/>
       <c r="K12" s="23" t="n"/>
       <c r="L12" s="23" t="n"/>
-      <c r="M12" s="24" t="n"/>
-      <c r="N12" s="24" t="n"/>
-      <c r="O12" s="24" t="n"/>
-      <c r="P12" s="24" t="n"/>
-      <c r="Q12" s="24" t="n"/>
+      <c r="M12" s="25" t="n"/>
+      <c r="N12" s="25" t="n"/>
+      <c r="O12" s="25" t="n"/>
+      <c r="P12" s="25" t="n"/>
+      <c r="Q12" s="25" t="n"/>
       <c r="S12">
         <f>IF(COUNTA($A12:$Q12)=0,0,IF(OR($B12="",$D12="",$F12="",$G12=""),1,0))</f>
         <v/>
@@ -2809,11 +2816,11 @@
       <c r="J13" s="23" t="n"/>
       <c r="K13" s="23" t="n"/>
       <c r="L13" s="23" t="n"/>
-      <c r="M13" s="24" t="n"/>
-      <c r="N13" s="24" t="n"/>
-      <c r="O13" s="24" t="n"/>
-      <c r="P13" s="24" t="n"/>
-      <c r="Q13" s="24" t="n"/>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="25" t="n"/>
+      <c r="O13" s="25" t="n"/>
+      <c r="P13" s="25" t="n"/>
+      <c r="Q13" s="25" t="n"/>
       <c r="S13">
         <f>IF(COUNTA($A13:$Q13)=0,0,IF(OR($B13="",$D13="",$F13="",$G13=""),1,0))</f>
         <v/>
@@ -2836,11 +2843,11 @@
       <c r="J14" s="23" t="n"/>
       <c r="K14" s="23" t="n"/>
       <c r="L14" s="23" t="n"/>
-      <c r="M14" s="24" t="n"/>
-      <c r="N14" s="24" t="n"/>
-      <c r="O14" s="24" t="n"/>
-      <c r="P14" s="24" t="n"/>
-      <c r="Q14" s="24" t="n"/>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="25" t="n"/>
+      <c r="O14" s="25" t="n"/>
+      <c r="P14" s="25" t="n"/>
+      <c r="Q14" s="25" t="n"/>
       <c r="S14">
         <f>IF(COUNTA($A14:$Q14)=0,0,IF(OR($B14="",$D14="",$F14="",$G14=""),1,0))</f>
         <v/>
@@ -2863,11 +2870,11 @@
       <c r="J15" s="23" t="n"/>
       <c r="K15" s="23" t="n"/>
       <c r="L15" s="23" t="n"/>
-      <c r="M15" s="24" t="n"/>
-      <c r="N15" s="24" t="n"/>
-      <c r="O15" s="24" t="n"/>
-      <c r="P15" s="24" t="n"/>
-      <c r="Q15" s="24" t="n"/>
+      <c r="M15" s="25" t="n"/>
+      <c r="N15" s="25" t="n"/>
+      <c r="O15" s="25" t="n"/>
+      <c r="P15" s="25" t="n"/>
+      <c r="Q15" s="25" t="n"/>
       <c r="S15">
         <f>IF(COUNTA($A15:$Q15)=0,0,IF(OR($B15="",$D15="",$F15="",$G15=""),1,0))</f>
         <v/>
@@ -2890,11 +2897,11 @@
       <c r="J16" s="23" t="n"/>
       <c r="K16" s="23" t="n"/>
       <c r="L16" s="23" t="n"/>
-      <c r="M16" s="24" t="n"/>
-      <c r="N16" s="24" t="n"/>
-      <c r="O16" s="24" t="n"/>
-      <c r="P16" s="24" t="n"/>
-      <c r="Q16" s="24" t="n"/>
+      <c r="M16" s="25" t="n"/>
+      <c r="N16" s="25" t="n"/>
+      <c r="O16" s="25" t="n"/>
+      <c r="P16" s="25" t="n"/>
+      <c r="Q16" s="25" t="n"/>
       <c r="S16">
         <f>IF(COUNTA($A16:$Q16)=0,0,IF(OR($B16="",$D16="",$F16="",$G16=""),1,0))</f>
         <v/>
@@ -2917,11 +2924,11 @@
       <c r="J17" s="23" t="n"/>
       <c r="K17" s="23" t="n"/>
       <c r="L17" s="23" t="n"/>
-      <c r="M17" s="24" t="n"/>
-      <c r="N17" s="24" t="n"/>
-      <c r="O17" s="24" t="n"/>
-      <c r="P17" s="24" t="n"/>
-      <c r="Q17" s="24" t="n"/>
+      <c r="M17" s="25" t="n"/>
+      <c r="N17" s="25" t="n"/>
+      <c r="O17" s="25" t="n"/>
+      <c r="P17" s="25" t="n"/>
+      <c r="Q17" s="25" t="n"/>
       <c r="S17">
         <f>IF(COUNTA($A17:$Q17)=0,0,IF(OR($B17="",$D17="",$F17="",$G17=""),1,0))</f>
         <v/>
@@ -2944,11 +2951,11 @@
       <c r="J18" s="23" t="n"/>
       <c r="K18" s="23" t="n"/>
       <c r="L18" s="23" t="n"/>
-      <c r="M18" s="24" t="n"/>
-      <c r="N18" s="24" t="n"/>
-      <c r="O18" s="24" t="n"/>
-      <c r="P18" s="24" t="n"/>
-      <c r="Q18" s="24" t="n"/>
+      <c r="M18" s="25" t="n"/>
+      <c r="N18" s="25" t="n"/>
+      <c r="O18" s="25" t="n"/>
+      <c r="P18" s="25" t="n"/>
+      <c r="Q18" s="25" t="n"/>
       <c r="S18">
         <f>IF(COUNTA($A18:$Q18)=0,0,IF(OR($B18="",$D18="",$F18="",$G18=""),1,0))</f>
         <v/>
@@ -2971,11 +2978,11 @@
       <c r="J19" s="23" t="n"/>
       <c r="K19" s="23" t="n"/>
       <c r="L19" s="23" t="n"/>
-      <c r="M19" s="24" t="n"/>
-      <c r="N19" s="24" t="n"/>
-      <c r="O19" s="24" t="n"/>
-      <c r="P19" s="24" t="n"/>
-      <c r="Q19" s="24" t="n"/>
+      <c r="M19" s="25" t="n"/>
+      <c r="N19" s="25" t="n"/>
+      <c r="O19" s="25" t="n"/>
+      <c r="P19" s="25" t="n"/>
+      <c r="Q19" s="25" t="n"/>
       <c r="S19">
         <f>IF(COUNTA($A19:$Q19)=0,0,IF(OR($B19="",$D19="",$F19="",$G19=""),1,0))</f>
         <v/>
@@ -2998,11 +3005,11 @@
       <c r="J20" s="23" t="n"/>
       <c r="K20" s="23" t="n"/>
       <c r="L20" s="23" t="n"/>
-      <c r="M20" s="24" t="n"/>
-      <c r="N20" s="24" t="n"/>
-      <c r="O20" s="24" t="n"/>
-      <c r="P20" s="24" t="n"/>
-      <c r="Q20" s="24" t="n"/>
+      <c r="M20" s="25" t="n"/>
+      <c r="N20" s="25" t="n"/>
+      <c r="O20" s="25" t="n"/>
+      <c r="P20" s="25" t="n"/>
+      <c r="Q20" s="25" t="n"/>
       <c r="S20">
         <f>IF(COUNTA($A20:$Q20)=0,0,IF(OR($B20="",$D20="",$F20="",$G20=""),1,0))</f>
         <v/>
@@ -3025,11 +3032,11 @@
       <c r="J21" s="23" t="n"/>
       <c r="K21" s="23" t="n"/>
       <c r="L21" s="23" t="n"/>
-      <c r="M21" s="24" t="n"/>
-      <c r="N21" s="24" t="n"/>
-      <c r="O21" s="24" t="n"/>
-      <c r="P21" s="24" t="n"/>
-      <c r="Q21" s="24" t="n"/>
+      <c r="M21" s="25" t="n"/>
+      <c r="N21" s="25" t="n"/>
+      <c r="O21" s="25" t="n"/>
+      <c r="P21" s="25" t="n"/>
+      <c r="Q21" s="25" t="n"/>
       <c r="S21">
         <f>IF(COUNTA($A21:$Q21)=0,0,IF(OR($B21="",$D21="",$F21="",$G21=""),1,0))</f>
         <v/>
@@ -3052,11 +3059,11 @@
       <c r="J22" s="23" t="n"/>
       <c r="K22" s="23" t="n"/>
       <c r="L22" s="23" t="n"/>
-      <c r="M22" s="24" t="n"/>
-      <c r="N22" s="24" t="n"/>
-      <c r="O22" s="24" t="n"/>
-      <c r="P22" s="24" t="n"/>
-      <c r="Q22" s="24" t="n"/>
+      <c r="M22" s="25" t="n"/>
+      <c r="N22" s="25" t="n"/>
+      <c r="O22" s="25" t="n"/>
+      <c r="P22" s="25" t="n"/>
+      <c r="Q22" s="25" t="n"/>
       <c r="S22">
         <f>IF(COUNTA($A22:$Q22)=0,0,IF(OR($B22="",$D22="",$F22="",$G22=""),1,0))</f>
         <v/>
@@ -3079,11 +3086,11 @@
       <c r="J23" s="23" t="n"/>
       <c r="K23" s="23" t="n"/>
       <c r="L23" s="23" t="n"/>
-      <c r="M23" s="24" t="n"/>
-      <c r="N23" s="24" t="n"/>
-      <c r="O23" s="24" t="n"/>
-      <c r="P23" s="24" t="n"/>
-      <c r="Q23" s="24" t="n"/>
+      <c r="M23" s="25" t="n"/>
+      <c r="N23" s="25" t="n"/>
+      <c r="O23" s="25" t="n"/>
+      <c r="P23" s="25" t="n"/>
+      <c r="Q23" s="25" t="n"/>
       <c r="S23">
         <f>IF(COUNTA($A23:$Q23)=0,0,IF(OR($B23="",$D23="",$F23="",$G23=""),1,0))</f>
         <v/>
@@ -3106,11 +3113,11 @@
       <c r="J24" s="23" t="n"/>
       <c r="K24" s="23" t="n"/>
       <c r="L24" s="23" t="n"/>
-      <c r="M24" s="24" t="n"/>
-      <c r="N24" s="24" t="n"/>
-      <c r="O24" s="24" t="n"/>
-      <c r="P24" s="24" t="n"/>
-      <c r="Q24" s="24" t="n"/>
+      <c r="M24" s="25" t="n"/>
+      <c r="N24" s="25" t="n"/>
+      <c r="O24" s="25" t="n"/>
+      <c r="P24" s="25" t="n"/>
+      <c r="Q24" s="25" t="n"/>
       <c r="S24">
         <f>IF(COUNTA($A24:$Q24)=0,0,IF(OR($B24="",$D24="",$F24="",$G24=""),1,0))</f>
         <v/>
@@ -3133,11 +3140,11 @@
       <c r="J25" s="23" t="n"/>
       <c r="K25" s="23" t="n"/>
       <c r="L25" s="23" t="n"/>
-      <c r="M25" s="24" t="n"/>
-      <c r="N25" s="24" t="n"/>
-      <c r="O25" s="24" t="n"/>
-      <c r="P25" s="24" t="n"/>
-      <c r="Q25" s="24" t="n"/>
+      <c r="M25" s="25" t="n"/>
+      <c r="N25" s="25" t="n"/>
+      <c r="O25" s="25" t="n"/>
+      <c r="P25" s="25" t="n"/>
+      <c r="Q25" s="25" t="n"/>
       <c r="S25">
         <f>IF(COUNTA($A25:$Q25)=0,0,IF(OR($B25="",$D25="",$F25="",$G25=""),1,0))</f>
         <v/>
@@ -3160,11 +3167,11 @@
       <c r="J26" s="23" t="n"/>
       <c r="K26" s="23" t="n"/>
       <c r="L26" s="23" t="n"/>
-      <c r="M26" s="24" t="n"/>
-      <c r="N26" s="24" t="n"/>
-      <c r="O26" s="24" t="n"/>
-      <c r="P26" s="24" t="n"/>
-      <c r="Q26" s="24" t="n"/>
+      <c r="M26" s="25" t="n"/>
+      <c r="N26" s="25" t="n"/>
+      <c r="O26" s="25" t="n"/>
+      <c r="P26" s="25" t="n"/>
+      <c r="Q26" s="25" t="n"/>
       <c r="S26">
         <f>IF(COUNTA($A26:$Q26)=0,0,IF(OR($B26="",$D26="",$F26="",$G26=""),1,0))</f>
         <v/>
@@ -3187,11 +3194,11 @@
       <c r="J27" s="23" t="n"/>
       <c r="K27" s="23" t="n"/>
       <c r="L27" s="23" t="n"/>
-      <c r="M27" s="24" t="n"/>
-      <c r="N27" s="24" t="n"/>
-      <c r="O27" s="24" t="n"/>
-      <c r="P27" s="24" t="n"/>
-      <c r="Q27" s="24" t="n"/>
+      <c r="M27" s="25" t="n"/>
+      <c r="N27" s="25" t="n"/>
+      <c r="O27" s="25" t="n"/>
+      <c r="P27" s="25" t="n"/>
+      <c r="Q27" s="25" t="n"/>
       <c r="S27">
         <f>IF(COUNTA($A27:$Q27)=0,0,IF(OR($B27="",$D27="",$F27="",$G27=""),1,0))</f>
         <v/>
@@ -3214,11 +3221,11 @@
       <c r="J28" s="23" t="n"/>
       <c r="K28" s="23" t="n"/>
       <c r="L28" s="23" t="n"/>
-      <c r="M28" s="24" t="n"/>
-      <c r="N28" s="24" t="n"/>
-      <c r="O28" s="24" t="n"/>
-      <c r="P28" s="24" t="n"/>
-      <c r="Q28" s="24" t="n"/>
+      <c r="M28" s="25" t="n"/>
+      <c r="N28" s="25" t="n"/>
+      <c r="O28" s="25" t="n"/>
+      <c r="P28" s="25" t="n"/>
+      <c r="Q28" s="25" t="n"/>
       <c r="S28">
         <f>IF(COUNTA($A28:$Q28)=0,0,IF(OR($B28="",$D28="",$F28="",$G28=""),1,0))</f>
         <v/>
@@ -3241,11 +3248,11 @@
       <c r="J29" s="23" t="n"/>
       <c r="K29" s="23" t="n"/>
       <c r="L29" s="23" t="n"/>
-      <c r="M29" s="24" t="n"/>
-      <c r="N29" s="24" t="n"/>
-      <c r="O29" s="24" t="n"/>
-      <c r="P29" s="24" t="n"/>
-      <c r="Q29" s="24" t="n"/>
+      <c r="M29" s="25" t="n"/>
+      <c r="N29" s="25" t="n"/>
+      <c r="O29" s="25" t="n"/>
+      <c r="P29" s="25" t="n"/>
+      <c r="Q29" s="25" t="n"/>
       <c r="S29">
         <f>IF(COUNTA($A29:$Q29)=0,0,IF(OR($B29="",$D29="",$F29="",$G29=""),1,0))</f>
         <v/>
@@ -3268,11 +3275,11 @@
       <c r="J30" s="23" t="n"/>
       <c r="K30" s="23" t="n"/>
       <c r="L30" s="23" t="n"/>
-      <c r="M30" s="24" t="n"/>
-      <c r="N30" s="24" t="n"/>
-      <c r="O30" s="24" t="n"/>
-      <c r="P30" s="24" t="n"/>
-      <c r="Q30" s="24" t="n"/>
+      <c r="M30" s="25" t="n"/>
+      <c r="N30" s="25" t="n"/>
+      <c r="O30" s="25" t="n"/>
+      <c r="P30" s="25" t="n"/>
+      <c r="Q30" s="25" t="n"/>
       <c r="S30">
         <f>IF(COUNTA($A30:$Q30)=0,0,IF(OR($B30="",$D30="",$F30="",$G30=""),1,0))</f>
         <v/>
@@ -3295,11 +3302,11 @@
       <c r="J31" s="23" t="n"/>
       <c r="K31" s="23" t="n"/>
       <c r="L31" s="23" t="n"/>
-      <c r="M31" s="24" t="n"/>
-      <c r="N31" s="24" t="n"/>
-      <c r="O31" s="24" t="n"/>
-      <c r="P31" s="24" t="n"/>
-      <c r="Q31" s="24" t="n"/>
+      <c r="M31" s="25" t="n"/>
+      <c r="N31" s="25" t="n"/>
+      <c r="O31" s="25" t="n"/>
+      <c r="P31" s="25" t="n"/>
+      <c r="Q31" s="25" t="n"/>
       <c r="S31">
         <f>IF(COUNTA($A31:$Q31)=0,0,IF(OR($B31="",$D31="",$F31="",$G31=""),1,0))</f>
         <v/>
@@ -3322,11 +3329,11 @@
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="23" t="n"/>
       <c r="L32" s="23" t="n"/>
-      <c r="M32" s="24" t="n"/>
-      <c r="N32" s="24" t="n"/>
-      <c r="O32" s="24" t="n"/>
-      <c r="P32" s="24" t="n"/>
-      <c r="Q32" s="24" t="n"/>
+      <c r="M32" s="25" t="n"/>
+      <c r="N32" s="25" t="n"/>
+      <c r="O32" s="25" t="n"/>
+      <c r="P32" s="25" t="n"/>
+      <c r="Q32" s="25" t="n"/>
       <c r="S32">
         <f>IF(COUNTA($A32:$Q32)=0,0,IF(OR($B32="",$D32="",$F32="",$G32=""),1,0))</f>
         <v/>
@@ -3349,11 +3356,11 @@
       <c r="J33" s="23" t="n"/>
       <c r="K33" s="23" t="n"/>
       <c r="L33" s="23" t="n"/>
-      <c r="M33" s="24" t="n"/>
-      <c r="N33" s="24" t="n"/>
-      <c r="O33" s="24" t="n"/>
-      <c r="P33" s="24" t="n"/>
-      <c r="Q33" s="24" t="n"/>
+      <c r="M33" s="25" t="n"/>
+      <c r="N33" s="25" t="n"/>
+      <c r="O33" s="25" t="n"/>
+      <c r="P33" s="25" t="n"/>
+      <c r="Q33" s="25" t="n"/>
       <c r="S33">
         <f>IF(COUNTA($A33:$Q33)=0,0,IF(OR($B33="",$D33="",$F33="",$G33=""),1,0))</f>
         <v/>
@@ -3376,11 +3383,11 @@
       <c r="J34" s="23" t="n"/>
       <c r="K34" s="23" t="n"/>
       <c r="L34" s="23" t="n"/>
-      <c r="M34" s="24" t="n"/>
-      <c r="N34" s="24" t="n"/>
-      <c r="O34" s="24" t="n"/>
-      <c r="P34" s="24" t="n"/>
-      <c r="Q34" s="24" t="n"/>
+      <c r="M34" s="25" t="n"/>
+      <c r="N34" s="25" t="n"/>
+      <c r="O34" s="25" t="n"/>
+      <c r="P34" s="25" t="n"/>
+      <c r="Q34" s="25" t="n"/>
       <c r="S34">
         <f>IF(COUNTA($A34:$Q34)=0,0,IF(OR($B34="",$D34="",$F34="",$G34=""),1,0))</f>
         <v/>
@@ -3403,11 +3410,11 @@
       <c r="J35" s="23" t="n"/>
       <c r="K35" s="23" t="n"/>
       <c r="L35" s="23" t="n"/>
-      <c r="M35" s="24" t="n"/>
-      <c r="N35" s="24" t="n"/>
-      <c r="O35" s="24" t="n"/>
-      <c r="P35" s="24" t="n"/>
-      <c r="Q35" s="24" t="n"/>
+      <c r="M35" s="25" t="n"/>
+      <c r="N35" s="25" t="n"/>
+      <c r="O35" s="25" t="n"/>
+      <c r="P35" s="25" t="n"/>
+      <c r="Q35" s="25" t="n"/>
       <c r="S35">
         <f>IF(COUNTA($A35:$Q35)=0,0,IF(OR($B35="",$D35="",$F35="",$G35=""),1,0))</f>
         <v/>
@@ -3430,11 +3437,11 @@
       <c r="J36" s="23" t="n"/>
       <c r="K36" s="23" t="n"/>
       <c r="L36" s="23" t="n"/>
-      <c r="M36" s="24" t="n"/>
-      <c r="N36" s="24" t="n"/>
-      <c r="O36" s="24" t="n"/>
-      <c r="P36" s="24" t="n"/>
-      <c r="Q36" s="24" t="n"/>
+      <c r="M36" s="25" t="n"/>
+      <c r="N36" s="25" t="n"/>
+      <c r="O36" s="25" t="n"/>
+      <c r="P36" s="25" t="n"/>
+      <c r="Q36" s="25" t="n"/>
       <c r="S36">
         <f>IF(COUNTA($A36:$Q36)=0,0,IF(OR($B36="",$D36="",$F36="",$G36=""),1,0))</f>
         <v/>
@@ -3457,11 +3464,11 @@
       <c r="J37" s="23" t="n"/>
       <c r="K37" s="23" t="n"/>
       <c r="L37" s="23" t="n"/>
-      <c r="M37" s="24" t="n"/>
-      <c r="N37" s="24" t="n"/>
-      <c r="O37" s="24" t="n"/>
-      <c r="P37" s="24" t="n"/>
-      <c r="Q37" s="24" t="n"/>
+      <c r="M37" s="25" t="n"/>
+      <c r="N37" s="25" t="n"/>
+      <c r="O37" s="25" t="n"/>
+      <c r="P37" s="25" t="n"/>
+      <c r="Q37" s="25" t="n"/>
       <c r="S37">
         <f>IF(COUNTA($A37:$Q37)=0,0,IF(OR($B37="",$D37="",$F37="",$G37=""),1,0))</f>
         <v/>
@@ -3484,11 +3491,11 @@
       <c r="J38" s="23" t="n"/>
       <c r="K38" s="23" t="n"/>
       <c r="L38" s="23" t="n"/>
-      <c r="M38" s="24" t="n"/>
-      <c r="N38" s="24" t="n"/>
-      <c r="O38" s="24" t="n"/>
-      <c r="P38" s="24" t="n"/>
-      <c r="Q38" s="24" t="n"/>
+      <c r="M38" s="25" t="n"/>
+      <c r="N38" s="25" t="n"/>
+      <c r="O38" s="25" t="n"/>
+      <c r="P38" s="25" t="n"/>
+      <c r="Q38" s="25" t="n"/>
       <c r="S38">
         <f>IF(COUNTA($A38:$Q38)=0,0,IF(OR($B38="",$D38="",$F38="",$G38=""),1,0))</f>
         <v/>
@@ -3511,11 +3518,11 @@
       <c r="J39" s="23" t="n"/>
       <c r="K39" s="23" t="n"/>
       <c r="L39" s="23" t="n"/>
-      <c r="M39" s="24" t="n"/>
-      <c r="N39" s="24" t="n"/>
-      <c r="O39" s="24" t="n"/>
-      <c r="P39" s="24" t="n"/>
-      <c r="Q39" s="24" t="n"/>
+      <c r="M39" s="25" t="n"/>
+      <c r="N39" s="25" t="n"/>
+      <c r="O39" s="25" t="n"/>
+      <c r="P39" s="25" t="n"/>
+      <c r="Q39" s="25" t="n"/>
       <c r="S39">
         <f>IF(COUNTA($A39:$Q39)=0,0,IF(OR($B39="",$D39="",$F39="",$G39=""),1,0))</f>
         <v/>
@@ -3538,11 +3545,11 @@
       <c r="J40" s="23" t="n"/>
       <c r="K40" s="23" t="n"/>
       <c r="L40" s="23" t="n"/>
-      <c r="M40" s="24" t="n"/>
-      <c r="N40" s="24" t="n"/>
-      <c r="O40" s="24" t="n"/>
-      <c r="P40" s="24" t="n"/>
-      <c r="Q40" s="24" t="n"/>
+      <c r="M40" s="25" t="n"/>
+      <c r="N40" s="25" t="n"/>
+      <c r="O40" s="25" t="n"/>
+      <c r="P40" s="25" t="n"/>
+      <c r="Q40" s="25" t="n"/>
       <c r="S40">
         <f>IF(COUNTA($A40:$Q40)=0,0,IF(OR($B40="",$D40="",$F40="",$G40=""),1,0))</f>
         <v/>
@@ -3565,11 +3572,11 @@
       <c r="J41" s="23" t="n"/>
       <c r="K41" s="23" t="n"/>
       <c r="L41" s="23" t="n"/>
-      <c r="M41" s="24" t="n"/>
-      <c r="N41" s="24" t="n"/>
-      <c r="O41" s="24" t="n"/>
-      <c r="P41" s="24" t="n"/>
-      <c r="Q41" s="24" t="n"/>
+      <c r="M41" s="25" t="n"/>
+      <c r="N41" s="25" t="n"/>
+      <c r="O41" s="25" t="n"/>
+      <c r="P41" s="25" t="n"/>
+      <c r="Q41" s="25" t="n"/>
       <c r="S41">
         <f>IF(COUNTA($A41:$Q41)=0,0,IF(OR($B41="",$D41="",$F41="",$G41=""),1,0))</f>
         <v/>
@@ -10707,8 +10714,8 @@
       <c r="D2" s="23" t="n"/>
       <c r="E2" s="23" t="n"/>
       <c r="F2" s="23" t="n"/>
-      <c r="G2" s="24" t="n"/>
-      <c r="H2" s="24" t="n"/>
+      <c r="G2" s="25" t="n"/>
+      <c r="H2" s="25" t="n"/>
       <c r="J2">
         <f>IF(COUNTA($A2:$H2)=0,0,IF(OR($B2="",$D2=""),1,0))</f>
         <v/>
@@ -10725,8 +10732,8 @@
       <c r="D3" s="23" t="n"/>
       <c r="E3" s="23" t="n"/>
       <c r="F3" s="23" t="n"/>
-      <c r="G3" s="24" t="n"/>
-      <c r="H3" s="24" t="n"/>
+      <c r="G3" s="25" t="n"/>
+      <c r="H3" s="25" t="n"/>
       <c r="J3">
         <f>IF(COUNTA($A3:$H3)=0,0,IF(OR($B3="",$D3=""),1,0))</f>
         <v/>
@@ -10743,8 +10750,8 @@
       <c r="D4" s="23" t="n"/>
       <c r="E4" s="23" t="n"/>
       <c r="F4" s="23" t="n"/>
-      <c r="G4" s="24" t="n"/>
-      <c r="H4" s="24" t="n"/>
+      <c r="G4" s="25" t="n"/>
+      <c r="H4" s="25" t="n"/>
       <c r="J4">
         <f>IF(COUNTA($A4:$H4)=0,0,IF(OR($B4="",$D4=""),1,0))</f>
         <v/>
@@ -10761,8 +10768,8 @@
       <c r="D5" s="23" t="n"/>
       <c r="E5" s="23" t="n"/>
       <c r="F5" s="23" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
+      <c r="H5" s="25" t="n"/>
       <c r="J5">
         <f>IF(COUNTA($A5:$H5)=0,0,IF(OR($B5="",$D5=""),1,0))</f>
         <v/>
@@ -10779,8 +10786,8 @@
       <c r="D6" s="23" t="n"/>
       <c r="E6" s="23" t="n"/>
       <c r="F6" s="23" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
+      <c r="G6" s="25" t="n"/>
+      <c r="H6" s="25" t="n"/>
       <c r="J6">
         <f>IF(COUNTA($A6:$H6)=0,0,IF(OR($B6="",$D6=""),1,0))</f>
         <v/>
@@ -10797,8 +10804,8 @@
       <c r="D7" s="23" t="n"/>
       <c r="E7" s="23" t="n"/>
       <c r="F7" s="23" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="24" t="n"/>
+      <c r="G7" s="25" t="n"/>
+      <c r="H7" s="25" t="n"/>
       <c r="J7">
         <f>IF(COUNTA($A7:$H7)=0,0,IF(OR($B7="",$D7=""),1,0))</f>
         <v/>
@@ -10815,8 +10822,8 @@
       <c r="D8" s="23" t="n"/>
       <c r="E8" s="23" t="n"/>
       <c r="F8" s="23" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="25" t="n"/>
       <c r="J8">
         <f>IF(COUNTA($A8:$H8)=0,0,IF(OR($B8="",$D8=""),1,0))</f>
         <v/>
@@ -10833,8 +10840,8 @@
       <c r="D9" s="23" t="n"/>
       <c r="E9" s="23" t="n"/>
       <c r="F9" s="23" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="24" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
       <c r="J9">
         <f>IF(COUNTA($A9:$H9)=0,0,IF(OR($B9="",$D9=""),1,0))</f>
         <v/>
@@ -10851,8 +10858,8 @@
       <c r="D10" s="23" t="n"/>
       <c r="E10" s="23" t="n"/>
       <c r="F10" s="23" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="24" t="n"/>
+      <c r="G10" s="25" t="n"/>
+      <c r="H10" s="25" t="n"/>
       <c r="J10">
         <f>IF(COUNTA($A10:$H10)=0,0,IF(OR($B10="",$D10=""),1,0))</f>
         <v/>
@@ -10869,8 +10876,8 @@
       <c r="D11" s="23" t="n"/>
       <c r="E11" s="23" t="n"/>
       <c r="F11" s="23" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="24" t="n"/>
+      <c r="G11" s="25" t="n"/>
+      <c r="H11" s="25" t="n"/>
       <c r="J11">
         <f>IF(COUNTA($A11:$H11)=0,0,IF(OR($B11="",$D11=""),1,0))</f>
         <v/>
@@ -10887,8 +10894,8 @@
       <c r="D12" s="23" t="n"/>
       <c r="E12" s="23" t="n"/>
       <c r="F12" s="23" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="H12" s="24" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="25" t="n"/>
       <c r="J12">
         <f>IF(COUNTA($A12:$H12)=0,0,IF(OR($B12="",$D12=""),1,0))</f>
         <v/>
@@ -10905,8 +10912,8 @@
       <c r="D13" s="23" t="n"/>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="23" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
       <c r="J13">
         <f>IF(COUNTA($A13:$H13)=0,0,IF(OR($B13="",$D13=""),1,0))</f>
         <v/>
@@ -10923,8 +10930,8 @@
       <c r="D14" s="23" t="n"/>
       <c r="E14" s="23" t="n"/>
       <c r="F14" s="23" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="24" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
       <c r="J14">
         <f>IF(COUNTA($A14:$H14)=0,0,IF(OR($B14="",$D14=""),1,0))</f>
         <v/>
@@ -10941,8 +10948,8 @@
       <c r="D15" s="23" t="n"/>
       <c r="E15" s="23" t="n"/>
       <c r="F15" s="23" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="24" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
       <c r="J15">
         <f>IF(COUNTA($A15:$H15)=0,0,IF(OR($B15="",$D15=""),1,0))</f>
         <v/>
@@ -10959,8 +10966,8 @@
       <c r="D16" s="23" t="n"/>
       <c r="E16" s="23" t="n"/>
       <c r="F16" s="23" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="24" t="n"/>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="25" t="n"/>
       <c r="J16">
         <f>IF(COUNTA($A16:$H16)=0,0,IF(OR($B16="",$D16=""),1,0))</f>
         <v/>
@@ -10977,8 +10984,8 @@
       <c r="D17" s="23" t="n"/>
       <c r="E17" s="23" t="n"/>
       <c r="F17" s="23" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="24" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
       <c r="J17">
         <f>IF(COUNTA($A17:$H17)=0,0,IF(OR($B17="",$D17=""),1,0))</f>
         <v/>
@@ -10995,8 +11002,8 @@
       <c r="D18" s="23" t="n"/>
       <c r="E18" s="23" t="n"/>
       <c r="F18" s="23" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
       <c r="J18">
         <f>IF(COUNTA($A18:$H18)=0,0,IF(OR($B18="",$D18=""),1,0))</f>
         <v/>
@@ -11013,8 +11020,8 @@
       <c r="D19" s="23" t="n"/>
       <c r="E19" s="23" t="n"/>
       <c r="F19" s="23" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
       <c r="J19">
         <f>IF(COUNTA($A19:$H19)=0,0,IF(OR($B19="",$D19=""),1,0))</f>
         <v/>
@@ -11031,8 +11038,8 @@
       <c r="D20" s="23" t="n"/>
       <c r="E20" s="23" t="n"/>
       <c r="F20" s="23" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="25" t="n"/>
       <c r="J20">
         <f>IF(COUNTA($A20:$H20)=0,0,IF(OR($B20="",$D20=""),1,0))</f>
         <v/>
@@ -11049,8 +11056,8 @@
       <c r="D21" s="23" t="n"/>
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
+      <c r="G21" s="25" t="n"/>
+      <c r="H21" s="25" t="n"/>
       <c r="J21">
         <f>IF(COUNTA($A21:$H21)=0,0,IF(OR($B21="",$D21=""),1,0))</f>
         <v/>
@@ -11067,8 +11074,8 @@
       <c r="D22" s="23" t="n"/>
       <c r="E22" s="23" t="n"/>
       <c r="F22" s="23" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24" t="n"/>
+      <c r="G22" s="25" t="n"/>
+      <c r="H22" s="25" t="n"/>
       <c r="J22">
         <f>IF(COUNTA($A22:$H22)=0,0,IF(OR($B22="",$D22=""),1,0))</f>
         <v/>
@@ -11085,8 +11092,8 @@
       <c r="D23" s="23" t="n"/>
       <c r="E23" s="23" t="n"/>
       <c r="F23" s="23" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="24" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="25" t="n"/>
       <c r="J23">
         <f>IF(COUNTA($A23:$H23)=0,0,IF(OR($B23="",$D23=""),1,0))</f>
         <v/>
@@ -11103,8 +11110,8 @@
       <c r="D24" s="23" t="n"/>
       <c r="E24" s="23" t="n"/>
       <c r="F24" s="23" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="24" t="n"/>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="25" t="n"/>
       <c r="J24">
         <f>IF(COUNTA($A24:$H24)=0,0,IF(OR($B24="",$D24=""),1,0))</f>
         <v/>
@@ -11121,8 +11128,8 @@
       <c r="D25" s="23" t="n"/>
       <c r="E25" s="23" t="n"/>
       <c r="F25" s="23" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="24" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
       <c r="J25">
         <f>IF(COUNTA($A25:$H25)=0,0,IF(OR($B25="",$D25=""),1,0))</f>
         <v/>
@@ -11139,8 +11146,8 @@
       <c r="D26" s="23" t="n"/>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
+      <c r="G26" s="25" t="n"/>
+      <c r="H26" s="25" t="n"/>
       <c r="J26">
         <f>IF(COUNTA($A26:$H26)=0,0,IF(OR($B26="",$D26=""),1,0))</f>
         <v/>
@@ -11157,8 +11164,8 @@
       <c r="D27" s="23" t="n"/>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="24" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="25" t="n"/>
       <c r="J27">
         <f>IF(COUNTA($A27:$H27)=0,0,IF(OR($B27="",$D27=""),1,0))</f>
         <v/>
@@ -11175,8 +11182,8 @@
       <c r="D28" s="23" t="n"/>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="24" t="n"/>
+      <c r="G28" s="25" t="n"/>
+      <c r="H28" s="25" t="n"/>
       <c r="J28">
         <f>IF(COUNTA($A28:$H28)=0,0,IF(OR($B28="",$D28=""),1,0))</f>
         <v/>
@@ -11193,8 +11200,8 @@
       <c r="D29" s="23" t="n"/>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="24" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="25" t="n"/>
       <c r="J29">
         <f>IF(COUNTA($A29:$H29)=0,0,IF(OR($B29="",$D29=""),1,0))</f>
         <v/>
@@ -11211,8 +11218,8 @@
       <c r="D30" s="23" t="n"/>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="24" t="n"/>
+      <c r="G30" s="25" t="n"/>
+      <c r="H30" s="25" t="n"/>
       <c r="J30">
         <f>IF(COUNTA($A30:$H30)=0,0,IF(OR($B30="",$D30=""),1,0))</f>
         <v/>
@@ -11229,8 +11236,8 @@
       <c r="D31" s="23" t="n"/>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="24" t="n"/>
+      <c r="G31" s="25" t="n"/>
+      <c r="H31" s="25" t="n"/>
       <c r="J31">
         <f>IF(COUNTA($A31:$H31)=0,0,IF(OR($B31="",$D31=""),1,0))</f>
         <v/>
@@ -11247,8 +11254,8 @@
       <c r="D32" s="23" t="n"/>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
+      <c r="G32" s="25" t="n"/>
+      <c r="H32" s="25" t="n"/>
       <c r="J32">
         <f>IF(COUNTA($A32:$H32)=0,0,IF(OR($B32="",$D32=""),1,0))</f>
         <v/>
@@ -11265,8 +11272,8 @@
       <c r="D33" s="23" t="n"/>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="24" t="n"/>
+      <c r="G33" s="25" t="n"/>
+      <c r="H33" s="25" t="n"/>
       <c r="J33">
         <f>IF(COUNTA($A33:$H33)=0,0,IF(OR($B33="",$D33=""),1,0))</f>
         <v/>
@@ -11283,8 +11290,8 @@
       <c r="D34" s="23" t="n"/>
       <c r="E34" s="23" t="n"/>
       <c r="F34" s="23" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
+      <c r="G34" s="25" t="n"/>
+      <c r="H34" s="25" t="n"/>
       <c r="J34">
         <f>IF(COUNTA($A34:$H34)=0,0,IF(OR($B34="",$D34=""),1,0))</f>
         <v/>
@@ -11301,8 +11308,8 @@
       <c r="D35" s="23" t="n"/>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="25" t="n"/>
       <c r="J35">
         <f>IF(COUNTA($A35:$H35)=0,0,IF(OR($B35="",$D35=""),1,0))</f>
         <v/>
@@ -11319,8 +11326,8 @@
       <c r="D36" s="23" t="n"/>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="25" t="n"/>
       <c r="J36">
         <f>IF(COUNTA($A36:$H36)=0,0,IF(OR($B36="",$D36=""),1,0))</f>
         <v/>
@@ -11337,8 +11344,8 @@
       <c r="D37" s="23" t="n"/>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
-      <c r="G37" s="24" t="n"/>
-      <c r="H37" s="24" t="n"/>
+      <c r="G37" s="25" t="n"/>
+      <c r="H37" s="25" t="n"/>
       <c r="J37">
         <f>IF(COUNTA($A37:$H37)=0,0,IF(OR($B37="",$D37=""),1,0))</f>
         <v/>
@@ -11355,8 +11362,8 @@
       <c r="D38" s="23" t="n"/>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="24" t="n"/>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="25" t="n"/>
       <c r="J38">
         <f>IF(COUNTA($A38:$H38)=0,0,IF(OR($B38="",$D38=""),1,0))</f>
         <v/>
@@ -11373,8 +11380,8 @@
       <c r="D39" s="23" t="n"/>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
       <c r="J39">
         <f>IF(COUNTA($A39:$H39)=0,0,IF(OR($B39="",$D39=""),1,0))</f>
         <v/>
@@ -11391,8 +11398,8 @@
       <c r="D40" s="23" t="n"/>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="25" t="n"/>
       <c r="J40">
         <f>IF(COUNTA($A40:$H40)=0,0,IF(OR($B40="",$D40=""),1,0))</f>
         <v/>
@@ -11409,8 +11416,8 @@
       <c r="D41" s="23" t="n"/>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="24" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
       <c r="J41">
         <f>IF(COUNTA($A41:$H41)=0,0,IF(OR($B41="",$D41=""),1,0))</f>
         <v/>
@@ -16198,8 +16205,8 @@
       <c r="D2" s="23" t="n"/>
       <c r="E2" s="23" t="n"/>
       <c r="F2" s="23" t="n"/>
-      <c r="G2" s="24" t="n"/>
-      <c r="H2" s="24" t="n"/>
+      <c r="G2" s="25" t="n"/>
+      <c r="H2" s="25" t="n"/>
       <c r="J2">
         <f>IF(COUNTA($A2:$H2)=0,0,IF(OR($B2="",$C2="",$E2=""),1,0))</f>
         <v/>
@@ -16216,8 +16223,8 @@
       <c r="D3" s="23" t="n"/>
       <c r="E3" s="23" t="n"/>
       <c r="F3" s="23" t="n"/>
-      <c r="G3" s="24" t="n"/>
-      <c r="H3" s="24" t="n"/>
+      <c r="G3" s="25" t="n"/>
+      <c r="H3" s="25" t="n"/>
       <c r="J3">
         <f>IF(COUNTA($A3:$H3)=0,0,IF(OR($B3="",$C3="",$E3=""),1,0))</f>
         <v/>
@@ -16234,8 +16241,8 @@
       <c r="D4" s="23" t="n"/>
       <c r="E4" s="23" t="n"/>
       <c r="F4" s="23" t="n"/>
-      <c r="G4" s="24" t="n"/>
-      <c r="H4" s="24" t="n"/>
+      <c r="G4" s="25" t="n"/>
+      <c r="H4" s="25" t="n"/>
       <c r="J4">
         <f>IF(COUNTA($A4:$H4)=0,0,IF(OR($B4="",$C4="",$E4=""),1,0))</f>
         <v/>
@@ -16252,8 +16259,8 @@
       <c r="D5" s="23" t="n"/>
       <c r="E5" s="23" t="n"/>
       <c r="F5" s="23" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
+      <c r="G5" s="25" t="n"/>
+      <c r="H5" s="25" t="n"/>
       <c r="J5">
         <f>IF(COUNTA($A5:$H5)=0,0,IF(OR($B5="",$C5="",$E5=""),1,0))</f>
         <v/>
@@ -16270,8 +16277,8 @@
       <c r="D6" s="23" t="n"/>
       <c r="E6" s="23" t="n"/>
       <c r="F6" s="23" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
+      <c r="G6" s="25" t="n"/>
+      <c r="H6" s="25" t="n"/>
       <c r="J6">
         <f>IF(COUNTA($A6:$H6)=0,0,IF(OR($B6="",$C6="",$E6=""),1,0))</f>
         <v/>
@@ -16288,8 +16295,8 @@
       <c r="D7" s="23" t="n"/>
       <c r="E7" s="23" t="n"/>
       <c r="F7" s="23" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="24" t="n"/>
+      <c r="G7" s="25" t="n"/>
+      <c r="H7" s="25" t="n"/>
       <c r="J7">
         <f>IF(COUNTA($A7:$H7)=0,0,IF(OR($B7="",$C7="",$E7=""),1,0))</f>
         <v/>
@@ -16306,8 +16313,8 @@
       <c r="D8" s="23" t="n"/>
       <c r="E8" s="23" t="n"/>
       <c r="F8" s="23" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="25" t="n"/>
       <c r="J8">
         <f>IF(COUNTA($A8:$H8)=0,0,IF(OR($B8="",$C8="",$E8=""),1,0))</f>
         <v/>
@@ -16324,8 +16331,8 @@
       <c r="D9" s="23" t="n"/>
       <c r="E9" s="23" t="n"/>
       <c r="F9" s="23" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="24" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
       <c r="J9">
         <f>IF(COUNTA($A9:$H9)=0,0,IF(OR($B9="",$C9="",$E9=""),1,0))</f>
         <v/>
@@ -16342,8 +16349,8 @@
       <c r="D10" s="23" t="n"/>
       <c r="E10" s="23" t="n"/>
       <c r="F10" s="23" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="24" t="n"/>
+      <c r="G10" s="25" t="n"/>
+      <c r="H10" s="25" t="n"/>
       <c r="J10">
         <f>IF(COUNTA($A10:$H10)=0,0,IF(OR($B10="",$C10="",$E10=""),1,0))</f>
         <v/>
@@ -16360,8 +16367,8 @@
       <c r="D11" s="23" t="n"/>
       <c r="E11" s="23" t="n"/>
       <c r="F11" s="23" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="24" t="n"/>
+      <c r="G11" s="25" t="n"/>
+      <c r="H11" s="25" t="n"/>
       <c r="J11">
         <f>IF(COUNTA($A11:$H11)=0,0,IF(OR($B11="",$C11="",$E11=""),1,0))</f>
         <v/>
@@ -16378,8 +16385,8 @@
       <c r="D12" s="23" t="n"/>
       <c r="E12" s="23" t="n"/>
       <c r="F12" s="23" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="H12" s="24" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="25" t="n"/>
       <c r="J12">
         <f>IF(COUNTA($A12:$H12)=0,0,IF(OR($B12="",$C12="",$E12=""),1,0))</f>
         <v/>
@@ -16396,8 +16403,8 @@
       <c r="D13" s="23" t="n"/>
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="23" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
       <c r="J13">
         <f>IF(COUNTA($A13:$H13)=0,0,IF(OR($B13="",$C13="",$E13=""),1,0))</f>
         <v/>
@@ -16414,8 +16421,8 @@
       <c r="D14" s="23" t="n"/>
       <c r="E14" s="23" t="n"/>
       <c r="F14" s="23" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="24" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
       <c r="J14">
         <f>IF(COUNTA($A14:$H14)=0,0,IF(OR($B14="",$C14="",$E14=""),1,0))</f>
         <v/>
@@ -16432,8 +16439,8 @@
       <c r="D15" s="23" t="n"/>
       <c r="E15" s="23" t="n"/>
       <c r="F15" s="23" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="24" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
       <c r="J15">
         <f>IF(COUNTA($A15:$H15)=0,0,IF(OR($B15="",$C15="",$E15=""),1,0))</f>
         <v/>
@@ -16450,8 +16457,8 @@
       <c r="D16" s="23" t="n"/>
       <c r="E16" s="23" t="n"/>
       <c r="F16" s="23" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="24" t="n"/>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="25" t="n"/>
       <c r="J16">
         <f>IF(COUNTA($A16:$H16)=0,0,IF(OR($B16="",$C16="",$E16=""),1,0))</f>
         <v/>
@@ -16468,8 +16475,8 @@
       <c r="D17" s="23" t="n"/>
       <c r="E17" s="23" t="n"/>
       <c r="F17" s="23" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="24" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
       <c r="J17">
         <f>IF(COUNTA($A17:$H17)=0,0,IF(OR($B17="",$C17="",$E17=""),1,0))</f>
         <v/>
@@ -16486,8 +16493,8 @@
       <c r="D18" s="23" t="n"/>
       <c r="E18" s="23" t="n"/>
       <c r="F18" s="23" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
       <c r="J18">
         <f>IF(COUNTA($A18:$H18)=0,0,IF(OR($B18="",$C18="",$E18=""),1,0))</f>
         <v/>
@@ -16504,8 +16511,8 @@
       <c r="D19" s="23" t="n"/>
       <c r="E19" s="23" t="n"/>
       <c r="F19" s="23" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
       <c r="J19">
         <f>IF(COUNTA($A19:$H19)=0,0,IF(OR($B19="",$C19="",$E19=""),1,0))</f>
         <v/>
@@ -16522,8 +16529,8 @@
       <c r="D20" s="23" t="n"/>
       <c r="E20" s="23" t="n"/>
       <c r="F20" s="23" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="25" t="n"/>
       <c r="J20">
         <f>IF(COUNTA($A20:$H20)=0,0,IF(OR($B20="",$C20="",$E20=""),1,0))</f>
         <v/>
@@ -16540,8 +16547,8 @@
       <c r="D21" s="23" t="n"/>
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
+      <c r="G21" s="25" t="n"/>
+      <c r="H21" s="25" t="n"/>
       <c r="J21">
         <f>IF(COUNTA($A21:$H21)=0,0,IF(OR($B21="",$C21="",$E21=""),1,0))</f>
         <v/>
@@ -16558,8 +16565,8 @@
       <c r="D22" s="23" t="n"/>
       <c r="E22" s="23" t="n"/>
       <c r="F22" s="23" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24" t="n"/>
+      <c r="G22" s="25" t="n"/>
+      <c r="H22" s="25" t="n"/>
       <c r="J22">
         <f>IF(COUNTA($A22:$H22)=0,0,IF(OR($B22="",$C22="",$E22=""),1,0))</f>
         <v/>
@@ -16576,8 +16583,8 @@
       <c r="D23" s="23" t="n"/>
       <c r="E23" s="23" t="n"/>
       <c r="F23" s="23" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="24" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="25" t="n"/>
       <c r="J23">
         <f>IF(COUNTA($A23:$H23)=0,0,IF(OR($B23="",$C23="",$E23=""),1,0))</f>
         <v/>
@@ -16594,8 +16601,8 @@
       <c r="D24" s="23" t="n"/>
       <c r="E24" s="23" t="n"/>
       <c r="F24" s="23" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="24" t="n"/>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="25" t="n"/>
       <c r="J24">
         <f>IF(COUNTA($A24:$H24)=0,0,IF(OR($B24="",$C24="",$E24=""),1,0))</f>
         <v/>
@@ -16612,8 +16619,8 @@
       <c r="D25" s="23" t="n"/>
       <c r="E25" s="23" t="n"/>
       <c r="F25" s="23" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="24" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
       <c r="J25">
         <f>IF(COUNTA($A25:$H25)=0,0,IF(OR($B25="",$C25="",$E25=""),1,0))</f>
         <v/>
@@ -16630,8 +16637,8 @@
       <c r="D26" s="23" t="n"/>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
+      <c r="G26" s="25" t="n"/>
+      <c r="H26" s="25" t="n"/>
       <c r="J26">
         <f>IF(COUNTA($A26:$H26)=0,0,IF(OR($B26="",$C26="",$E26=""),1,0))</f>
         <v/>
@@ -16648,8 +16655,8 @@
       <c r="D27" s="23" t="n"/>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="24" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="25" t="n"/>
       <c r="J27">
         <f>IF(COUNTA($A27:$H27)=0,0,IF(OR($B27="",$C27="",$E27=""),1,0))</f>
         <v/>
@@ -16666,8 +16673,8 @@
       <c r="D28" s="23" t="n"/>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="24" t="n"/>
+      <c r="G28" s="25" t="n"/>
+      <c r="H28" s="25" t="n"/>
       <c r="J28">
         <f>IF(COUNTA($A28:$H28)=0,0,IF(OR($B28="",$C28="",$E28=""),1,0))</f>
         <v/>
@@ -16684,8 +16691,8 @@
       <c r="D29" s="23" t="n"/>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="24" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="25" t="n"/>
       <c r="J29">
         <f>IF(COUNTA($A29:$H29)=0,0,IF(OR($B29="",$C29="",$E29=""),1,0))</f>
         <v/>
@@ -16702,8 +16709,8 @@
       <c r="D30" s="23" t="n"/>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="24" t="n"/>
+      <c r="G30" s="25" t="n"/>
+      <c r="H30" s="25" t="n"/>
       <c r="J30">
         <f>IF(COUNTA($A30:$H30)=0,0,IF(OR($B30="",$C30="",$E30=""),1,0))</f>
         <v/>
@@ -16720,8 +16727,8 @@
       <c r="D31" s="23" t="n"/>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="24" t="n"/>
+      <c r="G31" s="25" t="n"/>
+      <c r="H31" s="25" t="n"/>
       <c r="J31">
         <f>IF(COUNTA($A31:$H31)=0,0,IF(OR($B31="",$C31="",$E31=""),1,0))</f>
         <v/>
@@ -16738,8 +16745,8 @@
       <c r="D32" s="23" t="n"/>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
+      <c r="G32" s="25" t="n"/>
+      <c r="H32" s="25" t="n"/>
       <c r="J32">
         <f>IF(COUNTA($A32:$H32)=0,0,IF(OR($B32="",$C32="",$E32=""),1,0))</f>
         <v/>
@@ -16756,8 +16763,8 @@
       <c r="D33" s="23" t="n"/>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="24" t="n"/>
+      <c r="G33" s="25" t="n"/>
+      <c r="H33" s="25" t="n"/>
       <c r="J33">
         <f>IF(COUNTA($A33:$H33)=0,0,IF(OR($B33="",$C33="",$E33=""),1,0))</f>
         <v/>
@@ -16774,8 +16781,8 @@
       <c r="D34" s="23" t="n"/>
       <c r="E34" s="23" t="n"/>
       <c r="F34" s="23" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
+      <c r="G34" s="25" t="n"/>
+      <c r="H34" s="25" t="n"/>
       <c r="J34">
         <f>IF(COUNTA($A34:$H34)=0,0,IF(OR($B34="",$C34="",$E34=""),1,0))</f>
         <v/>
@@ -16792,8 +16799,8 @@
       <c r="D35" s="23" t="n"/>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="25" t="n"/>
       <c r="J35">
         <f>IF(COUNTA($A35:$H35)=0,0,IF(OR($B35="",$C35="",$E35=""),1,0))</f>
         <v/>
@@ -16810,8 +16817,8 @@
       <c r="D36" s="23" t="n"/>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="25" t="n"/>
       <c r="J36">
         <f>IF(COUNTA($A36:$H36)=0,0,IF(OR($B36="",$C36="",$E36=""),1,0))</f>
         <v/>
@@ -16828,8 +16835,8 @@
       <c r="D37" s="23" t="n"/>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
-      <c r="G37" s="24" t="n"/>
-      <c r="H37" s="24" t="n"/>
+      <c r="G37" s="25" t="n"/>
+      <c r="H37" s="25" t="n"/>
       <c r="J37">
         <f>IF(COUNTA($A37:$H37)=0,0,IF(OR($B37="",$C37="",$E37=""),1,0))</f>
         <v/>
@@ -16846,8 +16853,8 @@
       <c r="D38" s="23" t="n"/>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="24" t="n"/>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="25" t="n"/>
       <c r="J38">
         <f>IF(COUNTA($A38:$H38)=0,0,IF(OR($B38="",$C38="",$E38=""),1,0))</f>
         <v/>
@@ -16864,8 +16871,8 @@
       <c r="D39" s="23" t="n"/>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
       <c r="J39">
         <f>IF(COUNTA($A39:$H39)=0,0,IF(OR($B39="",$C39="",$E39=""),1,0))</f>
         <v/>
@@ -16882,8 +16889,8 @@
       <c r="D40" s="23" t="n"/>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="24" t="n"/>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="25" t="n"/>
       <c r="J40">
         <f>IF(COUNTA($A40:$H40)=0,0,IF(OR($B40="",$C40="",$E40=""),1,0))</f>
         <v/>
@@ -16900,8 +16907,8 @@
       <c r="D41" s="23" t="n"/>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="24" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
       <c r="J41">
         <f>IF(COUNTA($A41:$H41)=0,0,IF(OR($B41="",$C41="",$E41=""),1,0))</f>
         <v/>
@@ -21669,8 +21676,8 @@
       <c r="B2" s="23" t="n"/>
       <c r="C2" s="23" t="n"/>
       <c r="D2" s="23" t="n"/>
-      <c r="E2" s="24" t="n"/>
-      <c r="F2" s="24" t="n"/>
+      <c r="E2" s="25" t="n"/>
+      <c r="F2" s="25" t="n"/>
       <c r="H2">
         <f>IF(COUNTA($A2:$F2)=0,0,IF($B2="",1,0))</f>
         <v/>
@@ -21681,8 +21688,8 @@
       <c r="B3" s="23" t="n"/>
       <c r="C3" s="23" t="n"/>
       <c r="D3" s="23" t="n"/>
-      <c r="E3" s="24" t="n"/>
-      <c r="F3" s="24" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="25" t="n"/>
       <c r="H3">
         <f>IF(COUNTA($A3:$F3)=0,0,IF($B3="",1,0))</f>
         <v/>
@@ -21693,8 +21700,8 @@
       <c r="B4" s="23" t="n"/>
       <c r="C4" s="23" t="n"/>
       <c r="D4" s="23" t="n"/>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="24" t="n"/>
+      <c r="E4" s="25" t="n"/>
+      <c r="F4" s="25" t="n"/>
       <c r="H4">
         <f>IF(COUNTA($A4:$F4)=0,0,IF($B4="",1,0))</f>
         <v/>
@@ -21705,8 +21712,8 @@
       <c r="B5" s="23" t="n"/>
       <c r="C5" s="23" t="n"/>
       <c r="D5" s="23" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
+      <c r="E5" s="25" t="n"/>
+      <c r="F5" s="25" t="n"/>
       <c r="H5">
         <f>IF(COUNTA($A5:$F5)=0,0,IF($B5="",1,0))</f>
         <v/>
@@ -21717,8 +21724,8 @@
       <c r="B6" s="23" t="n"/>
       <c r="C6" s="23" t="n"/>
       <c r="D6" s="23" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="25" t="n"/>
       <c r="H6">
         <f>IF(COUNTA($A6:$F6)=0,0,IF($B6="",1,0))</f>
         <v/>
@@ -21729,8 +21736,8 @@
       <c r="B7" s="23" t="n"/>
       <c r="C7" s="23" t="n"/>
       <c r="D7" s="23" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
+      <c r="E7" s="25" t="n"/>
+      <c r="F7" s="25" t="n"/>
       <c r="H7">
         <f>IF(COUNTA($A7:$F7)=0,0,IF($B7="",1,0))</f>
         <v/>
@@ -21741,8 +21748,8 @@
       <c r="B8" s="23" t="n"/>
       <c r="C8" s="23" t="n"/>
       <c r="D8" s="23" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
       <c r="H8">
         <f>IF(COUNTA($A8:$F8)=0,0,IF($B8="",1,0))</f>
         <v/>
@@ -21753,8 +21760,8 @@
       <c r="B9" s="23" t="n"/>
       <c r="C9" s="23" t="n"/>
       <c r="D9" s="23" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="25" t="n"/>
       <c r="H9">
         <f>IF(COUNTA($A9:$F9)=0,0,IF($B9="",1,0))</f>
         <v/>
@@ -21765,8 +21772,8 @@
       <c r="B10" s="23" t="n"/>
       <c r="C10" s="23" t="n"/>
       <c r="D10" s="23" t="n"/>
-      <c r="E10" s="24" t="n"/>
-      <c r="F10" s="24" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="25" t="n"/>
       <c r="H10">
         <f>IF(COUNTA($A10:$F10)=0,0,IF($B10="",1,0))</f>
         <v/>
@@ -21777,8 +21784,8 @@
       <c r="B11" s="23" t="n"/>
       <c r="C11" s="23" t="n"/>
       <c r="D11" s="23" t="n"/>
-      <c r="E11" s="24" t="n"/>
-      <c r="F11" s="24" t="n"/>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="25" t="n"/>
       <c r="H11">
         <f>IF(COUNTA($A11:$F11)=0,0,IF($B11="",1,0))</f>
         <v/>
@@ -21789,8 +21796,8 @@
       <c r="B12" s="23" t="n"/>
       <c r="C12" s="23" t="n"/>
       <c r="D12" s="23" t="n"/>
-      <c r="E12" s="24" t="n"/>
-      <c r="F12" s="24" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="25" t="n"/>
       <c r="H12">
         <f>IF(COUNTA($A12:$F12)=0,0,IF($B12="",1,0))</f>
         <v/>
@@ -21801,8 +21808,8 @@
       <c r="B13" s="23" t="n"/>
       <c r="C13" s="23" t="n"/>
       <c r="D13" s="23" t="n"/>
-      <c r="E13" s="24" t="n"/>
-      <c r="F13" s="24" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
       <c r="H13">
         <f>IF(COUNTA($A13:$F13)=0,0,IF($B13="",1,0))</f>
         <v/>
@@ -21813,8 +21820,8 @@
       <c r="B14" s="23" t="n"/>
       <c r="C14" s="23" t="n"/>
       <c r="D14" s="23" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="24" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="25" t="n"/>
       <c r="H14">
         <f>IF(COUNTA($A14:$F14)=0,0,IF($B14="",1,0))</f>
         <v/>
@@ -21825,8 +21832,8 @@
       <c r="B15" s="23" t="n"/>
       <c r="C15" s="23" t="n"/>
       <c r="D15" s="23" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="24" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
       <c r="H15">
         <f>IF(COUNTA($A15:$F15)=0,0,IF($B15="",1,0))</f>
         <v/>
@@ -21837,8 +21844,8 @@
       <c r="B16" s="23" t="n"/>
       <c r="C16" s="23" t="n"/>
       <c r="D16" s="23" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="25" t="n"/>
       <c r="H16">
         <f>IF(COUNTA($A16:$F16)=0,0,IF($B16="",1,0))</f>
         <v/>
@@ -21849,8 +21856,8 @@
       <c r="B17" s="23" t="n"/>
       <c r="C17" s="23" t="n"/>
       <c r="D17" s="23" t="n"/>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="24" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
       <c r="H17">
         <f>IF(COUNTA($A17:$F17)=0,0,IF($B17="",1,0))</f>
         <v/>
@@ -21861,8 +21868,8 @@
       <c r="B18" s="23" t="n"/>
       <c r="C18" s="23" t="n"/>
       <c r="D18" s="23" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
       <c r="H18">
         <f>IF(COUNTA($A18:$F18)=0,0,IF($B18="",1,0))</f>
         <v/>
@@ -21873,8 +21880,8 @@
       <c r="B19" s="23" t="n"/>
       <c r="C19" s="23" t="n"/>
       <c r="D19" s="23" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
       <c r="H19">
         <f>IF(COUNTA($A19:$F19)=0,0,IF($B19="",1,0))</f>
         <v/>
@@ -21885,8 +21892,8 @@
       <c r="B20" s="23" t="n"/>
       <c r="C20" s="23" t="n"/>
       <c r="D20" s="23" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
       <c r="H20">
         <f>IF(COUNTA($A20:$F20)=0,0,IF($B20="",1,0))</f>
         <v/>
@@ -21897,8 +21904,8 @@
       <c r="B21" s="23" t="n"/>
       <c r="C21" s="23" t="n"/>
       <c r="D21" s="23" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
+      <c r="E21" s="25" t="n"/>
+      <c r="F21" s="25" t="n"/>
       <c r="H21">
         <f>IF(COUNTA($A21:$F21)=0,0,IF($B21="",1,0))</f>
         <v/>
@@ -21909,8 +21916,8 @@
       <c r="B22" s="23" t="n"/>
       <c r="C22" s="23" t="n"/>
       <c r="D22" s="23" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="25" t="n"/>
       <c r="H22">
         <f>IF(COUNTA($A22:$F22)=0,0,IF($B22="",1,0))</f>
         <v/>
@@ -21921,8 +21928,8 @@
       <c r="B23" s="23" t="n"/>
       <c r="C23" s="23" t="n"/>
       <c r="D23" s="23" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
       <c r="H23">
         <f>IF(COUNTA($A23:$F23)=0,0,IF($B23="",1,0))</f>
         <v/>
@@ -21933,8 +21940,8 @@
       <c r="B24" s="23" t="n"/>
       <c r="C24" s="23" t="n"/>
       <c r="D24" s="23" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="25" t="n"/>
       <c r="H24">
         <f>IF(COUNTA($A24:$F24)=0,0,IF($B24="",1,0))</f>
         <v/>
@@ -21945,8 +21952,8 @@
       <c r="B25" s="23" t="n"/>
       <c r="C25" s="23" t="n"/>
       <c r="D25" s="23" t="n"/>
-      <c r="E25" s="24" t="n"/>
-      <c r="F25" s="24" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
       <c r="H25">
         <f>IF(COUNTA($A25:$F25)=0,0,IF($B25="",1,0))</f>
         <v/>
@@ -21957,8 +21964,8 @@
       <c r="B26" s="23" t="n"/>
       <c r="C26" s="23" t="n"/>
       <c r="D26" s="23" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="25" t="n"/>
       <c r="H26">
         <f>IF(COUNTA($A26:$F26)=0,0,IF($B26="",1,0))</f>
         <v/>
@@ -21969,8 +21976,8 @@
       <c r="B27" s="23" t="n"/>
       <c r="C27" s="23" t="n"/>
       <c r="D27" s="23" t="n"/>
-      <c r="E27" s="24" t="n"/>
-      <c r="F27" s="24" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
       <c r="H27">
         <f>IF(COUNTA($A27:$F27)=0,0,IF($B27="",1,0))</f>
         <v/>
@@ -21981,8 +21988,8 @@
       <c r="B28" s="23" t="n"/>
       <c r="C28" s="23" t="n"/>
       <c r="D28" s="23" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
+      <c r="E28" s="25" t="n"/>
+      <c r="F28" s="25" t="n"/>
       <c r="H28">
         <f>IF(COUNTA($A28:$F28)=0,0,IF($B28="",1,0))</f>
         <v/>
@@ -21993,8 +22000,8 @@
       <c r="B29" s="23" t="n"/>
       <c r="C29" s="23" t="n"/>
       <c r="D29" s="23" t="n"/>
-      <c r="E29" s="24" t="n"/>
-      <c r="F29" s="24" t="n"/>
+      <c r="E29" s="25" t="n"/>
+      <c r="F29" s="25" t="n"/>
       <c r="H29">
         <f>IF(COUNTA($A29:$F29)=0,0,IF($B29="",1,0))</f>
         <v/>
@@ -22005,8 +22012,8 @@
       <c r="B30" s="23" t="n"/>
       <c r="C30" s="23" t="n"/>
       <c r="D30" s="23" t="n"/>
-      <c r="E30" s="24" t="n"/>
-      <c r="F30" s="24" t="n"/>
+      <c r="E30" s="25" t="n"/>
+      <c r="F30" s="25" t="n"/>
       <c r="H30">
         <f>IF(COUNTA($A30:$F30)=0,0,IF($B30="",1,0))</f>
         <v/>
@@ -22017,8 +22024,8 @@
       <c r="B31" s="23" t="n"/>
       <c r="C31" s="23" t="n"/>
       <c r="D31" s="23" t="n"/>
-      <c r="E31" s="24" t="n"/>
-      <c r="F31" s="24" t="n"/>
+      <c r="E31" s="25" t="n"/>
+      <c r="F31" s="25" t="n"/>
       <c r="H31">
         <f>IF(COUNTA($A31:$F31)=0,0,IF($B31="",1,0))</f>
         <v/>
@@ -22029,8 +22036,8 @@
       <c r="B32" s="23" t="n"/>
       <c r="C32" s="23" t="n"/>
       <c r="D32" s="23" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
+      <c r="E32" s="25" t="n"/>
+      <c r="F32" s="25" t="n"/>
       <c r="H32">
         <f>IF(COUNTA($A32:$F32)=0,0,IF($B32="",1,0))</f>
         <v/>
@@ -22041,8 +22048,8 @@
       <c r="B33" s="23" t="n"/>
       <c r="C33" s="23" t="n"/>
       <c r="D33" s="23" t="n"/>
-      <c r="E33" s="24" t="n"/>
-      <c r="F33" s="24" t="n"/>
+      <c r="E33" s="25" t="n"/>
+      <c r="F33" s="25" t="n"/>
       <c r="H33">
         <f>IF(COUNTA($A33:$F33)=0,0,IF($B33="",1,0))</f>
         <v/>
@@ -22053,8 +22060,8 @@
       <c r="B34" s="23" t="n"/>
       <c r="C34" s="23" t="n"/>
       <c r="D34" s="23" t="n"/>
-      <c r="E34" s="24" t="n"/>
-      <c r="F34" s="24" t="n"/>
+      <c r="E34" s="25" t="n"/>
+      <c r="F34" s="25" t="n"/>
       <c r="H34">
         <f>IF(COUNTA($A34:$F34)=0,0,IF($B34="",1,0))</f>
         <v/>
@@ -22065,8 +22072,8 @@
       <c r="B35" s="23" t="n"/>
       <c r="C35" s="23" t="n"/>
       <c r="D35" s="23" t="n"/>
-      <c r="E35" s="24" t="n"/>
-      <c r="F35" s="24" t="n"/>
+      <c r="E35" s="25" t="n"/>
+      <c r="F35" s="25" t="n"/>
       <c r="H35">
         <f>IF(COUNTA($A35:$F35)=0,0,IF($B35="",1,0))</f>
         <v/>
@@ -22077,8 +22084,8 @@
       <c r="B36" s="23" t="n"/>
       <c r="C36" s="23" t="n"/>
       <c r="D36" s="23" t="n"/>
-      <c r="E36" s="24" t="n"/>
-      <c r="F36" s="24" t="n"/>
+      <c r="E36" s="25" t="n"/>
+      <c r="F36" s="25" t="n"/>
       <c r="H36">
         <f>IF(COUNTA($A36:$F36)=0,0,IF($B36="",1,0))</f>
         <v/>
@@ -22089,8 +22096,8 @@
       <c r="B37" s="23" t="n"/>
       <c r="C37" s="23" t="n"/>
       <c r="D37" s="23" t="n"/>
-      <c r="E37" s="24" t="n"/>
-      <c r="F37" s="24" t="n"/>
+      <c r="E37" s="25" t="n"/>
+      <c r="F37" s="25" t="n"/>
       <c r="H37">
         <f>IF(COUNTA($A37:$F37)=0,0,IF($B37="",1,0))</f>
         <v/>
@@ -22101,8 +22108,8 @@
       <c r="B38" s="23" t="n"/>
       <c r="C38" s="23" t="n"/>
       <c r="D38" s="23" t="n"/>
-      <c r="E38" s="24" t="n"/>
-      <c r="F38" s="24" t="n"/>
+      <c r="E38" s="25" t="n"/>
+      <c r="F38" s="25" t="n"/>
       <c r="H38">
         <f>IF(COUNTA($A38:$F38)=0,0,IF($B38="",1,0))</f>
         <v/>
@@ -22113,8 +22120,8 @@
       <c r="B39" s="23" t="n"/>
       <c r="C39" s="23" t="n"/>
       <c r="D39" s="23" t="n"/>
-      <c r="E39" s="24" t="n"/>
-      <c r="F39" s="24" t="n"/>
+      <c r="E39" s="25" t="n"/>
+      <c r="F39" s="25" t="n"/>
       <c r="H39">
         <f>IF(COUNTA($A39:$F39)=0,0,IF($B39="",1,0))</f>
         <v/>
@@ -22125,8 +22132,8 @@
       <c r="B40" s="23" t="n"/>
       <c r="C40" s="23" t="n"/>
       <c r="D40" s="23" t="n"/>
-      <c r="E40" s="24" t="n"/>
-      <c r="F40" s="24" t="n"/>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="25" t="n"/>
       <c r="H40">
         <f>IF(COUNTA($A40:$F40)=0,0,IF($B40="",1,0))</f>
         <v/>
@@ -22137,8 +22144,8 @@
       <c r="B41" s="23" t="n"/>
       <c r="C41" s="23" t="n"/>
       <c r="D41" s="23" t="n"/>
-      <c r="E41" s="24" t="n"/>
-      <c r="F41" s="24" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
       <c r="H41">
         <f>IF(COUNTA($A41:$F41)=0,0,IF($B41="",1,0))</f>
         <v/>

</xml_diff>